<commit_message>
refactor: update profile test flow to sign in before each test case; enhance combobox handling and validation messages
</commit_message>
<xml_diff>
--- a/test_data/data.xlsx
+++ b/test_data/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Linh\Đồ án\DATN\linky-testing\test_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8DF485D-1840-4C31-8269-BE1139780C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{125EE1DE-CD48-4F8B-904C-1D9ABB76B920}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sign_up" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="91">
   <si>
     <t>email</t>
   </si>
@@ -293,6 +293,12 @@
   </si>
   <si>
     <t>Invalid characters in input.</t>
+  </si>
+  <si>
+    <t>No country found.</t>
+  </si>
+  <si>
+    <t>Hà Nội</t>
   </si>
 </sst>
 </file>
@@ -348,7 +354,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -432,12 +438,53 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -530,11 +577,23 @@
     <xf numFmtId="3" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1054,7 +1113,7 @@
       </c>
     </row>
     <row r="13" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="34" t="s">
+      <c r="A13" s="32" t="s">
         <v>84</v>
       </c>
       <c r="B13" s="5" t="s">
@@ -1071,7 +1130,7 @@
       </c>
     </row>
     <row r="14" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="34" t="s">
+      <c r="A14" s="32" t="s">
         <v>75</v>
       </c>
       <c r="B14" s="5" t="s">
@@ -1241,10 +1300,10 @@
       </c>
     </row>
     <row r="9" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="32" t="s">
         <v>68</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="32" t="s">
         <v>64</v>
       </c>
       <c r="C9" s="6">
@@ -1308,6 +1367,10 @@
     <row r="23" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="24" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A9" r:id="rId1" xr:uid="{B0378A5B-FB57-4231-B0C5-A900FF98D36F}"/>
+    <hyperlink ref="B9" r:id="rId2" xr:uid="{BF442790-459F-4CBD-ABC3-BE5F56B93638}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1317,7 +1380,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.1640625" style="20" bestFit="1" customWidth="1"/>
@@ -1514,27 +1577,23 @@
     </row>
     <row r="13" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="16"/>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="D13" s="16"/>
+      <c r="B13" s="35"/>
+      <c r="C13" s="38" t="s">
+        <v>90</v>
+      </c>
+      <c r="D13" s="36"/>
       <c r="E13" s="17"/>
       <c r="F13" s="16"/>
       <c r="G13" s="16"/>
       <c r="H13" s="16" t="s">
-        <v>38</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="B14" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="C14" s="16" t="s">
-        <v>41</v>
+      <c r="A14" s="16"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="37" t="s">
+        <v>42</v>
       </c>
       <c r="D14" s="16"/>
       <c r="E14" s="17"/>
@@ -1546,37 +1605,41 @@
     </row>
     <row r="15" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="16" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="C15" s="16"/>
+        <v>43</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>41</v>
+      </c>
       <c r="D15" s="16"/>
       <c r="E15" s="17"/>
       <c r="F15" s="16"/>
       <c r="G15" s="16"/>
-      <c r="H15" s="9" t="s">
-        <v>40</v>
+      <c r="H15" s="16" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="B16" s="16"/>
+      <c r="A16" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>39</v>
+      </c>
       <c r="C16" s="16"/>
       <c r="D16" s="16"/>
       <c r="E16" s="17"/>
       <c r="F16" s="16"/>
       <c r="G16" s="16"/>
       <c r="H16" s="9" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B17" s="16"/>
       <c r="C17" s="16"/>
@@ -1584,13 +1647,13 @@
       <c r="E17" s="17"/>
       <c r="F17" s="16"/>
       <c r="G17" s="16"/>
-      <c r="H17" s="16" t="s">
-        <v>38</v>
+      <c r="H17" s="9" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B18" s="16"/>
       <c r="C18" s="16"/>
@@ -1598,22 +1661,22 @@
       <c r="E18" s="17"/>
       <c r="F18" s="16"/>
       <c r="G18" s="16"/>
-      <c r="H18" s="9" t="s">
-        <v>88</v>
+      <c r="H18" s="16" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="16"/>
+      <c r="A19" s="9" t="s">
+        <v>48</v>
+      </c>
       <c r="B19" s="16"/>
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
-      <c r="E19" s="17" t="s">
-        <v>49</v>
-      </c>
+      <c r="E19" s="17"/>
       <c r="F19" s="16"/>
       <c r="G19" s="16"/>
       <c r="H19" s="9" t="s">
-        <v>50</v>
+        <v>88</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -1621,10 +1684,10 @@
       <c r="B20" s="16"/>
       <c r="C20" s="16"/>
       <c r="D20" s="16"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="16" t="s">
-        <v>51</v>
-      </c>
+      <c r="E20" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="F20" s="16"/>
       <c r="G20" s="16"/>
       <c r="H20" s="9" t="s">
         <v>50</v>
@@ -1635,11 +1698,9 @@
       <c r="B21" s="16"/>
       <c r="C21" s="16"/>
       <c r="D21" s="16"/>
-      <c r="E21" s="17">
-        <v>37956</v>
-      </c>
-      <c r="F21" s="19" t="s">
-        <v>52</v>
+      <c r="E21" s="17"/>
+      <c r="F21" s="16" t="s">
+        <v>51</v>
       </c>
       <c r="G21" s="16"/>
       <c r="H21" s="9" t="s">
@@ -1651,11 +1712,11 @@
       <c r="B22" s="16"/>
       <c r="C22" s="16"/>
       <c r="D22" s="16"/>
-      <c r="E22" s="17" t="s">
-        <v>53</v>
-      </c>
-      <c r="F22" s="16" t="s">
-        <v>53</v>
+      <c r="E22" s="17">
+        <v>37956</v>
+      </c>
+      <c r="F22" s="19" t="s">
+        <v>52</v>
       </c>
       <c r="G22" s="16"/>
       <c r="H22" s="9" t="s">
@@ -1668,12 +1729,14 @@
       <c r="C23" s="16"/>
       <c r="D23" s="16"/>
       <c r="E23" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="F23" s="16"/>
+        <v>53</v>
+      </c>
+      <c r="F23" s="16" t="s">
+        <v>53</v>
+      </c>
       <c r="G23" s="16"/>
       <c r="H23" s="9" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -1681,13 +1744,13 @@
       <c r="B24" s="16"/>
       <c r="C24" s="16"/>
       <c r="D24" s="16"/>
-      <c r="E24" s="17">
-        <v>36526</v>
+      <c r="E24" s="17" t="s">
+        <v>54</v>
       </c>
       <c r="F24" s="16"/>
       <c r="G24" s="16"/>
       <c r="H24" s="9" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -1695,13 +1758,13 @@
       <c r="B25" s="16"/>
       <c r="C25" s="16"/>
       <c r="D25" s="16"/>
-      <c r="E25" s="17"/>
+      <c r="E25" s="17">
+        <v>36526</v>
+      </c>
       <c r="F25" s="16"/>
-      <c r="G25" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="H25" s="16" t="s">
-        <v>57</v>
+      <c r="G25" s="16"/>
+      <c r="H25" s="9" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -1712,7 +1775,7 @@
       <c r="E26" s="17"/>
       <c r="F26" s="16"/>
       <c r="G26" s="16" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H26" s="16" t="s">
         <v>57</v>
@@ -1726,7 +1789,7 @@
       <c r="E27" s="17"/>
       <c r="F27" s="16"/>
       <c r="G27" s="16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H27" s="16" t="s">
         <v>57</v>
@@ -1740,10 +1803,10 @@
       <c r="E28" s="17"/>
       <c r="F28" s="16"/>
       <c r="G28" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="H28" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
+      </c>
+      <c r="H28" s="16" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -1753,8 +1816,12 @@
       <c r="D29" s="16"/>
       <c r="E29" s="17"/>
       <c r="F29" s="16"/>
-      <c r="G29" s="16"/>
-      <c r="H29" s="16"/>
+      <c r="G29" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="H29" s="7" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="30" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="16"/>
@@ -1835,6 +1902,16 @@
       <c r="F37" s="16"/>
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
+    </row>
+    <row r="38" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="16"/>
+      <c r="B38" s="16"/>
+      <c r="C38" s="16"/>
+      <c r="D38" s="16"/>
+      <c r="E38" s="17"/>
+      <c r="F38" s="16"/>
+      <c r="G38" s="16"/>
+      <c r="H38" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1884,9 +1961,9 @@
       </c>
       <c r="H1" s="4"/>
       <c r="I1" s="4"/>
-      <c r="J1" s="32"/>
-      <c r="K1" s="33"/>
-      <c r="L1" s="33"/>
+      <c r="J1" s="33"/>
+      <c r="K1" s="34"/>
+      <c r="L1" s="34"/>
       <c r="M1" s="4"/>
       <c r="N1" s="4"/>
       <c r="O1" s="4"/>
@@ -2101,9 +2178,9 @@
       <c r="G2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="33"/>
-      <c r="K2" s="33"/>
-      <c r="L2" s="33"/>
+      <c r="J2" s="34"/>
+      <c r="K2" s="34"/>
+      <c r="L2" s="34"/>
     </row>
     <row r="3" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
@@ -2121,9 +2198,9 @@
       <c r="G3" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="33"/>
-      <c r="K3" s="33"/>
-      <c r="L3" s="33"/>
+      <c r="J3" s="34"/>
+      <c r="K3" s="34"/>
+      <c r="L3" s="34"/>
     </row>
     <row r="4" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
@@ -2147,9 +2224,9 @@
       <c r="G4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="J4" s="33"/>
-      <c r="K4" s="33"/>
-      <c r="L4" s="33"/>
+      <c r="J4" s="34"/>
+      <c r="K4" s="34"/>
+      <c r="L4" s="34"/>
     </row>
     <row r="5" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
@@ -2173,9 +2250,9 @@
       <c r="G5" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="J5" s="33"/>
-      <c r="K5" s="33"/>
-      <c r="L5" s="33"/>
+      <c r="J5" s="34"/>
+      <c r="K5" s="34"/>
+      <c r="L5" s="34"/>
     </row>
     <row r="6" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
@@ -2199,9 +2276,9 @@
       <c r="G6" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="J6" s="33"/>
-      <c r="K6" s="33"/>
-      <c r="L6" s="33"/>
+      <c r="J6" s="34"/>
+      <c r="K6" s="34"/>
+      <c r="L6" s="34"/>
     </row>
     <row r="7" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
@@ -2225,9 +2302,9 @@
       <c r="G7" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="J7" s="33"/>
-      <c r="K7" s="33"/>
-      <c r="L7" s="33"/>
+      <c r="J7" s="34"/>
+      <c r="K7" s="34"/>
+      <c r="L7" s="34"/>
     </row>
     <row r="8" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
@@ -2251,9 +2328,9 @@
       <c r="G8" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="J8" s="33"/>
-      <c r="K8" s="33"/>
-      <c r="L8" s="33"/>
+      <c r="J8" s="34"/>
+      <c r="K8" s="34"/>
+      <c r="L8" s="34"/>
     </row>
     <row r="9" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
@@ -2277,9 +2354,9 @@
       <c r="G9" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="J9" s="33"/>
-      <c r="K9" s="33"/>
-      <c r="L9" s="33"/>
+      <c r="J9" s="34"/>
+      <c r="K9" s="34"/>
+      <c r="L9" s="34"/>
     </row>
     <row r="10" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
@@ -2303,9 +2380,9 @@
       <c r="G10" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="J10" s="33"/>
-      <c r="K10" s="33"/>
-      <c r="L10" s="33"/>
+      <c r="J10" s="34"/>
+      <c r="K10" s="34"/>
+      <c r="L10" s="34"/>
     </row>
     <row r="11" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
@@ -2329,9 +2406,9 @@
       <c r="G11" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="J11" s="33"/>
-      <c r="K11" s="33"/>
-      <c r="L11" s="33"/>
+      <c r="J11" s="34"/>
+      <c r="K11" s="34"/>
+      <c r="L11" s="34"/>
     </row>
     <row r="12" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
@@ -2355,9 +2432,9 @@
       <c r="G12" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="J12" s="33"/>
-      <c r="K12" s="33"/>
-      <c r="L12" s="33"/>
+      <c r="J12" s="34"/>
+      <c r="K12" s="34"/>
+      <c r="L12" s="34"/>
     </row>
     <row r="13" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
@@ -2381,9 +2458,9 @@
       <c r="G13" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="J13" s="33"/>
-      <c r="K13" s="33"/>
-      <c r="L13" s="33"/>
+      <c r="J13" s="34"/>
+      <c r="K13" s="34"/>
+      <c r="L13" s="34"/>
     </row>
     <row r="14" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
@@ -2407,9 +2484,9 @@
       <c r="G14" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="J14" s="33"/>
-      <c r="K14" s="33"/>
-      <c r="L14" s="33"/>
+      <c r="J14" s="34"/>
+      <c r="K14" s="34"/>
+      <c r="L14" s="34"/>
     </row>
     <row r="15" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
@@ -2433,9 +2510,9 @@
       <c r="G15" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="J15" s="33"/>
-      <c r="K15" s="33"/>
-      <c r="L15" s="33"/>
+      <c r="J15" s="34"/>
+      <c r="K15" s="34"/>
+      <c r="L15" s="34"/>
     </row>
     <row r="16" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
@@ -2459,9 +2536,9 @@
       <c r="G16" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="J16" s="33"/>
-      <c r="K16" s="33"/>
-      <c r="L16" s="33"/>
+      <c r="J16" s="34"/>
+      <c r="K16" s="34"/>
+      <c r="L16" s="34"/>
     </row>
     <row r="17" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
@@ -2485,9 +2562,9 @@
       <c r="G17" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="J17" s="33"/>
-      <c r="K17" s="33"/>
-      <c r="L17" s="33"/>
+      <c r="J17" s="34"/>
+      <c r="K17" s="34"/>
+      <c r="L17" s="34"/>
     </row>
     <row r="18" spans="1:12" ht="83.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
@@ -2511,919 +2588,919 @@
       <c r="G18" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="J18" s="33"/>
-      <c r="K18" s="33"/>
-      <c r="L18" s="33"/>
+      <c r="J18" s="34"/>
+      <c r="K18" s="34"/>
+      <c r="L18" s="34"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J19" s="33"/>
-      <c r="K19" s="33"/>
-      <c r="L19" s="33"/>
+      <c r="J19" s="34"/>
+      <c r="K19" s="34"/>
+      <c r="L19" s="34"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J20" s="33"/>
-      <c r="K20" s="33"/>
-      <c r="L20" s="33"/>
+      <c r="J20" s="34"/>
+      <c r="K20" s="34"/>
+      <c r="L20" s="34"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J21" s="33"/>
-      <c r="K21" s="33"/>
-      <c r="L21" s="33"/>
+      <c r="J21" s="34"/>
+      <c r="K21" s="34"/>
+      <c r="L21" s="34"/>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J22" s="33"/>
-      <c r="K22" s="33"/>
-      <c r="L22" s="33"/>
+      <c r="J22" s="34"/>
+      <c r="K22" s="34"/>
+      <c r="L22" s="34"/>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J23" s="33"/>
-      <c r="K23" s="33"/>
-      <c r="L23" s="33"/>
+      <c r="J23" s="34"/>
+      <c r="K23" s="34"/>
+      <c r="L23" s="34"/>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J24" s="33"/>
-      <c r="K24" s="33"/>
-      <c r="L24" s="33"/>
+      <c r="J24" s="34"/>
+      <c r="K24" s="34"/>
+      <c r="L24" s="34"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J25" s="33"/>
-      <c r="K25" s="33"/>
-      <c r="L25" s="33"/>
+      <c r="J25" s="34"/>
+      <c r="K25" s="34"/>
+      <c r="L25" s="34"/>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J26" s="33"/>
-      <c r="K26" s="33"/>
-      <c r="L26" s="33"/>
+      <c r="J26" s="34"/>
+      <c r="K26" s="34"/>
+      <c r="L26" s="34"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J27" s="33"/>
-      <c r="K27" s="33"/>
-      <c r="L27" s="33"/>
+      <c r="J27" s="34"/>
+      <c r="K27" s="34"/>
+      <c r="L27" s="34"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J28" s="33"/>
-      <c r="K28" s="33"/>
-      <c r="L28" s="33"/>
+      <c r="J28" s="34"/>
+      <c r="K28" s="34"/>
+      <c r="L28" s="34"/>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J29" s="33"/>
-      <c r="K29" s="33"/>
-      <c r="L29" s="33"/>
+      <c r="J29" s="34"/>
+      <c r="K29" s="34"/>
+      <c r="L29" s="34"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J30" s="33"/>
-      <c r="K30" s="33"/>
-      <c r="L30" s="33"/>
+      <c r="J30" s="34"/>
+      <c r="K30" s="34"/>
+      <c r="L30" s="34"/>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J31" s="33"/>
-      <c r="K31" s="33"/>
-      <c r="L31" s="33"/>
+      <c r="J31" s="34"/>
+      <c r="K31" s="34"/>
+      <c r="L31" s="34"/>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J32" s="33"/>
-      <c r="K32" s="33"/>
-      <c r="L32" s="33"/>
+      <c r="J32" s="34"/>
+      <c r="K32" s="34"/>
+      <c r="L32" s="34"/>
     </row>
     <row r="33" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J33" s="33"/>
-      <c r="K33" s="33"/>
-      <c r="L33" s="33"/>
+      <c r="J33" s="34"/>
+      <c r="K33" s="34"/>
+      <c r="L33" s="34"/>
     </row>
     <row r="34" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J34" s="33"/>
-      <c r="K34" s="33"/>
-      <c r="L34" s="33"/>
+      <c r="J34" s="34"/>
+      <c r="K34" s="34"/>
+      <c r="L34" s="34"/>
     </row>
     <row r="35" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J35" s="33"/>
-      <c r="K35" s="33"/>
-      <c r="L35" s="33"/>
+      <c r="J35" s="34"/>
+      <c r="K35" s="34"/>
+      <c r="L35" s="34"/>
     </row>
     <row r="36" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J36" s="33"/>
-      <c r="K36" s="33"/>
-      <c r="L36" s="33"/>
+      <c r="J36" s="34"/>
+      <c r="K36" s="34"/>
+      <c r="L36" s="34"/>
     </row>
     <row r="37" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J37" s="33"/>
-      <c r="K37" s="33"/>
-      <c r="L37" s="33"/>
+      <c r="J37" s="34"/>
+      <c r="K37" s="34"/>
+      <c r="L37" s="34"/>
     </row>
     <row r="38" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J38" s="33"/>
-      <c r="K38" s="33"/>
-      <c r="L38" s="33"/>
+      <c r="J38" s="34"/>
+      <c r="K38" s="34"/>
+      <c r="L38" s="34"/>
     </row>
     <row r="39" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J39" s="33"/>
-      <c r="K39" s="33"/>
-      <c r="L39" s="33"/>
+      <c r="J39" s="34"/>
+      <c r="K39" s="34"/>
+      <c r="L39" s="34"/>
     </row>
     <row r="40" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J40" s="33"/>
-      <c r="K40" s="33"/>
-      <c r="L40" s="33"/>
+      <c r="J40" s="34"/>
+      <c r="K40" s="34"/>
+      <c r="L40" s="34"/>
     </row>
     <row r="41" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J41" s="33"/>
-      <c r="K41" s="33"/>
-      <c r="L41" s="33"/>
+      <c r="J41" s="34"/>
+      <c r="K41" s="34"/>
+      <c r="L41" s="34"/>
     </row>
     <row r="42" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J42" s="33"/>
-      <c r="K42" s="33"/>
-      <c r="L42" s="33"/>
+      <c r="J42" s="34"/>
+      <c r="K42" s="34"/>
+      <c r="L42" s="34"/>
     </row>
     <row r="43" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J43" s="33"/>
-      <c r="K43" s="33"/>
-      <c r="L43" s="33"/>
+      <c r="J43" s="34"/>
+      <c r="K43" s="34"/>
+      <c r="L43" s="34"/>
     </row>
     <row r="44" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J44" s="33"/>
-      <c r="K44" s="33"/>
-      <c r="L44" s="33"/>
+      <c r="J44" s="34"/>
+      <c r="K44" s="34"/>
+      <c r="L44" s="34"/>
     </row>
     <row r="45" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J45" s="33"/>
-      <c r="K45" s="33"/>
-      <c r="L45" s="33"/>
+      <c r="J45" s="34"/>
+      <c r="K45" s="34"/>
+      <c r="L45" s="34"/>
     </row>
     <row r="46" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J46" s="33"/>
-      <c r="K46" s="33"/>
-      <c r="L46" s="33"/>
+      <c r="J46" s="34"/>
+      <c r="K46" s="34"/>
+      <c r="L46" s="34"/>
     </row>
     <row r="47" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J47" s="33"/>
-      <c r="K47" s="33"/>
-      <c r="L47" s="33"/>
+      <c r="J47" s="34"/>
+      <c r="K47" s="34"/>
+      <c r="L47" s="34"/>
     </row>
     <row r="48" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J48" s="33"/>
-      <c r="K48" s="33"/>
-      <c r="L48" s="33"/>
+      <c r="J48" s="34"/>
+      <c r="K48" s="34"/>
+      <c r="L48" s="34"/>
     </row>
     <row r="49" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J49" s="33"/>
-      <c r="K49" s="33"/>
-      <c r="L49" s="33"/>
+      <c r="J49" s="34"/>
+      <c r="K49" s="34"/>
+      <c r="L49" s="34"/>
     </row>
     <row r="50" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J50" s="33"/>
-      <c r="K50" s="33"/>
-      <c r="L50" s="33"/>
+      <c r="J50" s="34"/>
+      <c r="K50" s="34"/>
+      <c r="L50" s="34"/>
     </row>
     <row r="51" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J51" s="33"/>
-      <c r="K51" s="33"/>
-      <c r="L51" s="33"/>
+      <c r="J51" s="34"/>
+      <c r="K51" s="34"/>
+      <c r="L51" s="34"/>
     </row>
     <row r="52" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J52" s="33"/>
-      <c r="K52" s="33"/>
-      <c r="L52" s="33"/>
+      <c r="J52" s="34"/>
+      <c r="K52" s="34"/>
+      <c r="L52" s="34"/>
     </row>
     <row r="53" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J53" s="33"/>
-      <c r="K53" s="33"/>
-      <c r="L53" s="33"/>
+      <c r="J53" s="34"/>
+      <c r="K53" s="34"/>
+      <c r="L53" s="34"/>
     </row>
     <row r="54" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J54" s="33"/>
-      <c r="K54" s="33"/>
-      <c r="L54" s="33"/>
+      <c r="J54" s="34"/>
+      <c r="K54" s="34"/>
+      <c r="L54" s="34"/>
     </row>
     <row r="55" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J55" s="33"/>
-      <c r="K55" s="33"/>
-      <c r="L55" s="33"/>
+      <c r="J55" s="34"/>
+      <c r="K55" s="34"/>
+      <c r="L55" s="34"/>
     </row>
     <row r="56" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J56" s="33"/>
-      <c r="K56" s="33"/>
-      <c r="L56" s="33"/>
+      <c r="J56" s="34"/>
+      <c r="K56" s="34"/>
+      <c r="L56" s="34"/>
     </row>
     <row r="57" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J57" s="33"/>
-      <c r="K57" s="33"/>
-      <c r="L57" s="33"/>
+      <c r="J57" s="34"/>
+      <c r="K57" s="34"/>
+      <c r="L57" s="34"/>
     </row>
     <row r="58" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J58" s="33"/>
-      <c r="K58" s="33"/>
-      <c r="L58" s="33"/>
+      <c r="J58" s="34"/>
+      <c r="K58" s="34"/>
+      <c r="L58" s="34"/>
     </row>
     <row r="59" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J59" s="33"/>
-      <c r="K59" s="33"/>
-      <c r="L59" s="33"/>
+      <c r="J59" s="34"/>
+      <c r="K59" s="34"/>
+      <c r="L59" s="34"/>
     </row>
     <row r="60" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J60" s="33"/>
-      <c r="K60" s="33"/>
-      <c r="L60" s="33"/>
+      <c r="J60" s="34"/>
+      <c r="K60" s="34"/>
+      <c r="L60" s="34"/>
     </row>
     <row r="61" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J61" s="33"/>
-      <c r="K61" s="33"/>
-      <c r="L61" s="33"/>
+      <c r="J61" s="34"/>
+      <c r="K61" s="34"/>
+      <c r="L61" s="34"/>
     </row>
     <row r="62" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J62" s="33"/>
-      <c r="K62" s="33"/>
-      <c r="L62" s="33"/>
+      <c r="J62" s="34"/>
+      <c r="K62" s="34"/>
+      <c r="L62" s="34"/>
     </row>
     <row r="63" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J63" s="33"/>
-      <c r="K63" s="33"/>
-      <c r="L63" s="33"/>
+      <c r="J63" s="34"/>
+      <c r="K63" s="34"/>
+      <c r="L63" s="34"/>
     </row>
     <row r="64" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J64" s="33"/>
-      <c r="K64" s="33"/>
-      <c r="L64" s="33"/>
+      <c r="J64" s="34"/>
+      <c r="K64" s="34"/>
+      <c r="L64" s="34"/>
     </row>
     <row r="65" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J65" s="33"/>
-      <c r="K65" s="33"/>
-      <c r="L65" s="33"/>
+      <c r="J65" s="34"/>
+      <c r="K65" s="34"/>
+      <c r="L65" s="34"/>
     </row>
     <row r="66" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J66" s="33"/>
-      <c r="K66" s="33"/>
-      <c r="L66" s="33"/>
+      <c r="J66" s="34"/>
+      <c r="K66" s="34"/>
+      <c r="L66" s="34"/>
     </row>
     <row r="67" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J67" s="33"/>
-      <c r="K67" s="33"/>
-      <c r="L67" s="33"/>
+      <c r="J67" s="34"/>
+      <c r="K67" s="34"/>
+      <c r="L67" s="34"/>
     </row>
     <row r="68" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J68" s="33"/>
-      <c r="K68" s="33"/>
-      <c r="L68" s="33"/>
+      <c r="J68" s="34"/>
+      <c r="K68" s="34"/>
+      <c r="L68" s="34"/>
     </row>
     <row r="69" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J69" s="33"/>
-      <c r="K69" s="33"/>
-      <c r="L69" s="33"/>
+      <c r="J69" s="34"/>
+      <c r="K69" s="34"/>
+      <c r="L69" s="34"/>
     </row>
     <row r="70" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J70" s="33"/>
-      <c r="K70" s="33"/>
-      <c r="L70" s="33"/>
+      <c r="J70" s="34"/>
+      <c r="K70" s="34"/>
+      <c r="L70" s="34"/>
     </row>
     <row r="71" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J71" s="33"/>
-      <c r="K71" s="33"/>
-      <c r="L71" s="33"/>
+      <c r="J71" s="34"/>
+      <c r="K71" s="34"/>
+      <c r="L71" s="34"/>
     </row>
     <row r="72" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J72" s="33"/>
-      <c r="K72" s="33"/>
-      <c r="L72" s="33"/>
+      <c r="J72" s="34"/>
+      <c r="K72" s="34"/>
+      <c r="L72" s="34"/>
     </row>
     <row r="73" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J73" s="33"/>
-      <c r="K73" s="33"/>
-      <c r="L73" s="33"/>
+      <c r="J73" s="34"/>
+      <c r="K73" s="34"/>
+      <c r="L73" s="34"/>
     </row>
     <row r="74" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J74" s="33"/>
-      <c r="K74" s="33"/>
-      <c r="L74" s="33"/>
+      <c r="J74" s="34"/>
+      <c r="K74" s="34"/>
+      <c r="L74" s="34"/>
     </row>
     <row r="75" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J75" s="33"/>
-      <c r="K75" s="33"/>
-      <c r="L75" s="33"/>
+      <c r="J75" s="34"/>
+      <c r="K75" s="34"/>
+      <c r="L75" s="34"/>
     </row>
     <row r="76" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J76" s="33"/>
-      <c r="K76" s="33"/>
-      <c r="L76" s="33"/>
+      <c r="J76" s="34"/>
+      <c r="K76" s="34"/>
+      <c r="L76" s="34"/>
     </row>
     <row r="77" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J77" s="33"/>
-      <c r="K77" s="33"/>
-      <c r="L77" s="33"/>
+      <c r="J77" s="34"/>
+      <c r="K77" s="34"/>
+      <c r="L77" s="34"/>
     </row>
     <row r="78" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J78" s="33"/>
-      <c r="K78" s="33"/>
-      <c r="L78" s="33"/>
+      <c r="J78" s="34"/>
+      <c r="K78" s="34"/>
+      <c r="L78" s="34"/>
     </row>
     <row r="79" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J79" s="33"/>
-      <c r="K79" s="33"/>
-      <c r="L79" s="33"/>
+      <c r="J79" s="34"/>
+      <c r="K79" s="34"/>
+      <c r="L79" s="34"/>
     </row>
     <row r="80" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J80" s="33"/>
-      <c r="K80" s="33"/>
-      <c r="L80" s="33"/>
+      <c r="J80" s="34"/>
+      <c r="K80" s="34"/>
+      <c r="L80" s="34"/>
     </row>
     <row r="81" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J81" s="33"/>
-      <c r="K81" s="33"/>
-      <c r="L81" s="33"/>
+      <c r="J81" s="34"/>
+      <c r="K81" s="34"/>
+      <c r="L81" s="34"/>
     </row>
     <row r="82" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J82" s="33"/>
-      <c r="K82" s="33"/>
-      <c r="L82" s="33"/>
+      <c r="J82" s="34"/>
+      <c r="K82" s="34"/>
+      <c r="L82" s="34"/>
     </row>
     <row r="83" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J83" s="33"/>
-      <c r="K83" s="33"/>
-      <c r="L83" s="33"/>
+      <c r="J83" s="34"/>
+      <c r="K83" s="34"/>
+      <c r="L83" s="34"/>
     </row>
     <row r="84" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J84" s="33"/>
-      <c r="K84" s="33"/>
-      <c r="L84" s="33"/>
+      <c r="J84" s="34"/>
+      <c r="K84" s="34"/>
+      <c r="L84" s="34"/>
     </row>
     <row r="85" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J85" s="33"/>
-      <c r="K85" s="33"/>
-      <c r="L85" s="33"/>
+      <c r="J85" s="34"/>
+      <c r="K85" s="34"/>
+      <c r="L85" s="34"/>
     </row>
     <row r="86" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J86" s="33"/>
-      <c r="K86" s="33"/>
-      <c r="L86" s="33"/>
+      <c r="J86" s="34"/>
+      <c r="K86" s="34"/>
+      <c r="L86" s="34"/>
     </row>
     <row r="87" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J87" s="33"/>
-      <c r="K87" s="33"/>
-      <c r="L87" s="33"/>
+      <c r="J87" s="34"/>
+      <c r="K87" s="34"/>
+      <c r="L87" s="34"/>
     </row>
     <row r="88" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J88" s="33"/>
-      <c r="K88" s="33"/>
-      <c r="L88" s="33"/>
+      <c r="J88" s="34"/>
+      <c r="K88" s="34"/>
+      <c r="L88" s="34"/>
     </row>
     <row r="89" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J89" s="33"/>
-      <c r="K89" s="33"/>
-      <c r="L89" s="33"/>
+      <c r="J89" s="34"/>
+      <c r="K89" s="34"/>
+      <c r="L89" s="34"/>
     </row>
     <row r="90" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J90" s="33"/>
-      <c r="K90" s="33"/>
-      <c r="L90" s="33"/>
+      <c r="J90" s="34"/>
+      <c r="K90" s="34"/>
+      <c r="L90" s="34"/>
     </row>
     <row r="91" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J91" s="33"/>
-      <c r="K91" s="33"/>
-      <c r="L91" s="33"/>
+      <c r="J91" s="34"/>
+      <c r="K91" s="34"/>
+      <c r="L91" s="34"/>
     </row>
     <row r="92" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J92" s="33"/>
-      <c r="K92" s="33"/>
-      <c r="L92" s="33"/>
+      <c r="J92" s="34"/>
+      <c r="K92" s="34"/>
+      <c r="L92" s="34"/>
     </row>
     <row r="93" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J93" s="33"/>
-      <c r="K93" s="33"/>
-      <c r="L93" s="33"/>
+      <c r="J93" s="34"/>
+      <c r="K93" s="34"/>
+      <c r="L93" s="34"/>
     </row>
     <row r="94" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J94" s="33"/>
-      <c r="K94" s="33"/>
-      <c r="L94" s="33"/>
+      <c r="J94" s="34"/>
+      <c r="K94" s="34"/>
+      <c r="L94" s="34"/>
     </row>
     <row r="95" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J95" s="33"/>
-      <c r="K95" s="33"/>
-      <c r="L95" s="33"/>
+      <c r="J95" s="34"/>
+      <c r="K95" s="34"/>
+      <c r="L95" s="34"/>
     </row>
     <row r="96" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J96" s="33"/>
-      <c r="K96" s="33"/>
-      <c r="L96" s="33"/>
+      <c r="J96" s="34"/>
+      <c r="K96" s="34"/>
+      <c r="L96" s="34"/>
     </row>
     <row r="97" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J97" s="33"/>
-      <c r="K97" s="33"/>
-      <c r="L97" s="33"/>
+      <c r="J97" s="34"/>
+      <c r="K97" s="34"/>
+      <c r="L97" s="34"/>
     </row>
     <row r="98" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J98" s="33"/>
-      <c r="K98" s="33"/>
-      <c r="L98" s="33"/>
+      <c r="J98" s="34"/>
+      <c r="K98" s="34"/>
+      <c r="L98" s="34"/>
     </row>
     <row r="99" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J99" s="33"/>
-      <c r="K99" s="33"/>
-      <c r="L99" s="33"/>
+      <c r="J99" s="34"/>
+      <c r="K99" s="34"/>
+      <c r="L99" s="34"/>
     </row>
     <row r="100" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J100" s="33"/>
-      <c r="K100" s="33"/>
-      <c r="L100" s="33"/>
+      <c r="J100" s="34"/>
+      <c r="K100" s="34"/>
+      <c r="L100" s="34"/>
     </row>
     <row r="101" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J101" s="33"/>
-      <c r="K101" s="33"/>
-      <c r="L101" s="33"/>
+      <c r="J101" s="34"/>
+      <c r="K101" s="34"/>
+      <c r="L101" s="34"/>
     </row>
     <row r="102" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J102" s="33"/>
-      <c r="K102" s="33"/>
-      <c r="L102" s="33"/>
+      <c r="J102" s="34"/>
+      <c r="K102" s="34"/>
+      <c r="L102" s="34"/>
     </row>
     <row r="103" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J103" s="33"/>
-      <c r="K103" s="33"/>
-      <c r="L103" s="33"/>
+      <c r="J103" s="34"/>
+      <c r="K103" s="34"/>
+      <c r="L103" s="34"/>
     </row>
     <row r="104" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J104" s="33"/>
-      <c r="K104" s="33"/>
-      <c r="L104" s="33"/>
+      <c r="J104" s="34"/>
+      <c r="K104" s="34"/>
+      <c r="L104" s="34"/>
     </row>
     <row r="105" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J105" s="33"/>
-      <c r="K105" s="33"/>
-      <c r="L105" s="33"/>
+      <c r="J105" s="34"/>
+      <c r="K105" s="34"/>
+      <c r="L105" s="34"/>
     </row>
     <row r="106" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J106" s="33"/>
-      <c r="K106" s="33"/>
-      <c r="L106" s="33"/>
+      <c r="J106" s="34"/>
+      <c r="K106" s="34"/>
+      <c r="L106" s="34"/>
     </row>
     <row r="107" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J107" s="33"/>
-      <c r="K107" s="33"/>
-      <c r="L107" s="33"/>
+      <c r="J107" s="34"/>
+      <c r="K107" s="34"/>
+      <c r="L107" s="34"/>
     </row>
     <row r="108" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J108" s="33"/>
-      <c r="K108" s="33"/>
-      <c r="L108" s="33"/>
+      <c r="J108" s="34"/>
+      <c r="K108" s="34"/>
+      <c r="L108" s="34"/>
     </row>
     <row r="109" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J109" s="33"/>
-      <c r="K109" s="33"/>
-      <c r="L109" s="33"/>
+      <c r="J109" s="34"/>
+      <c r="K109" s="34"/>
+      <c r="L109" s="34"/>
     </row>
     <row r="110" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J110" s="33"/>
-      <c r="K110" s="33"/>
-      <c r="L110" s="33"/>
+      <c r="J110" s="34"/>
+      <c r="K110" s="34"/>
+      <c r="L110" s="34"/>
     </row>
     <row r="111" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J111" s="33"/>
-      <c r="K111" s="33"/>
-      <c r="L111" s="33"/>
+      <c r="J111" s="34"/>
+      <c r="K111" s="34"/>
+      <c r="L111" s="34"/>
     </row>
     <row r="112" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J112" s="33"/>
-      <c r="K112" s="33"/>
-      <c r="L112" s="33"/>
+      <c r="J112" s="34"/>
+      <c r="K112" s="34"/>
+      <c r="L112" s="34"/>
     </row>
     <row r="113" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J113" s="33"/>
-      <c r="K113" s="33"/>
-      <c r="L113" s="33"/>
+      <c r="J113" s="34"/>
+      <c r="K113" s="34"/>
+      <c r="L113" s="34"/>
     </row>
     <row r="114" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J114" s="33"/>
-      <c r="K114" s="33"/>
-      <c r="L114" s="33"/>
+      <c r="J114" s="34"/>
+      <c r="K114" s="34"/>
+      <c r="L114" s="34"/>
     </row>
     <row r="115" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J115" s="33"/>
-      <c r="K115" s="33"/>
-      <c r="L115" s="33"/>
+      <c r="J115" s="34"/>
+      <c r="K115" s="34"/>
+      <c r="L115" s="34"/>
     </row>
     <row r="116" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J116" s="33"/>
-      <c r="K116" s="33"/>
-      <c r="L116" s="33"/>
+      <c r="J116" s="34"/>
+      <c r="K116" s="34"/>
+      <c r="L116" s="34"/>
     </row>
     <row r="117" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J117" s="33"/>
-      <c r="K117" s="33"/>
-      <c r="L117" s="33"/>
+      <c r="J117" s="34"/>
+      <c r="K117" s="34"/>
+      <c r="L117" s="34"/>
     </row>
     <row r="118" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J118" s="33"/>
-      <c r="K118" s="33"/>
-      <c r="L118" s="33"/>
+      <c r="J118" s="34"/>
+      <c r="K118" s="34"/>
+      <c r="L118" s="34"/>
     </row>
     <row r="119" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J119" s="33"/>
-      <c r="K119" s="33"/>
-      <c r="L119" s="33"/>
+      <c r="J119" s="34"/>
+      <c r="K119" s="34"/>
+      <c r="L119" s="34"/>
     </row>
     <row r="120" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J120" s="33"/>
-      <c r="K120" s="33"/>
-      <c r="L120" s="33"/>
+      <c r="J120" s="34"/>
+      <c r="K120" s="34"/>
+      <c r="L120" s="34"/>
     </row>
     <row r="121" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J121" s="33"/>
-      <c r="K121" s="33"/>
-      <c r="L121" s="33"/>
+      <c r="J121" s="34"/>
+      <c r="K121" s="34"/>
+      <c r="L121" s="34"/>
     </row>
     <row r="122" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J122" s="33"/>
-      <c r="K122" s="33"/>
-      <c r="L122" s="33"/>
+      <c r="J122" s="34"/>
+      <c r="K122" s="34"/>
+      <c r="L122" s="34"/>
     </row>
     <row r="123" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J123" s="33"/>
-      <c r="K123" s="33"/>
-      <c r="L123" s="33"/>
+      <c r="J123" s="34"/>
+      <c r="K123" s="34"/>
+      <c r="L123" s="34"/>
     </row>
     <row r="124" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J124" s="33"/>
-      <c r="K124" s="33"/>
-      <c r="L124" s="33"/>
+      <c r="J124" s="34"/>
+      <c r="K124" s="34"/>
+      <c r="L124" s="34"/>
     </row>
     <row r="125" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J125" s="33"/>
-      <c r="K125" s="33"/>
-      <c r="L125" s="33"/>
+      <c r="J125" s="34"/>
+      <c r="K125" s="34"/>
+      <c r="L125" s="34"/>
     </row>
     <row r="126" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J126" s="33"/>
-      <c r="K126" s="33"/>
-      <c r="L126" s="33"/>
+      <c r="J126" s="34"/>
+      <c r="K126" s="34"/>
+      <c r="L126" s="34"/>
     </row>
     <row r="127" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J127" s="33"/>
-      <c r="K127" s="33"/>
-      <c r="L127" s="33"/>
+      <c r="J127" s="34"/>
+      <c r="K127" s="34"/>
+      <c r="L127" s="34"/>
     </row>
     <row r="128" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J128" s="33"/>
-      <c r="K128" s="33"/>
-      <c r="L128" s="33"/>
+      <c r="J128" s="34"/>
+      <c r="K128" s="34"/>
+      <c r="L128" s="34"/>
     </row>
     <row r="129" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J129" s="33"/>
-      <c r="K129" s="33"/>
-      <c r="L129" s="33"/>
+      <c r="J129" s="34"/>
+      <c r="K129" s="34"/>
+      <c r="L129" s="34"/>
     </row>
     <row r="130" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J130" s="33"/>
-      <c r="K130" s="33"/>
-      <c r="L130" s="33"/>
+      <c r="J130" s="34"/>
+      <c r="K130" s="34"/>
+      <c r="L130" s="34"/>
     </row>
     <row r="131" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J131" s="33"/>
-      <c r="K131" s="33"/>
-      <c r="L131" s="33"/>
+      <c r="J131" s="34"/>
+      <c r="K131" s="34"/>
+      <c r="L131" s="34"/>
     </row>
     <row r="132" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J132" s="33"/>
-      <c r="K132" s="33"/>
-      <c r="L132" s="33"/>
+      <c r="J132" s="34"/>
+      <c r="K132" s="34"/>
+      <c r="L132" s="34"/>
     </row>
     <row r="133" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J133" s="33"/>
-      <c r="K133" s="33"/>
-      <c r="L133" s="33"/>
+      <c r="J133" s="34"/>
+      <c r="K133" s="34"/>
+      <c r="L133" s="34"/>
     </row>
     <row r="134" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J134" s="33"/>
-      <c r="K134" s="33"/>
-      <c r="L134" s="33"/>
+      <c r="J134" s="34"/>
+      <c r="K134" s="34"/>
+      <c r="L134" s="34"/>
     </row>
     <row r="135" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J135" s="33"/>
-      <c r="K135" s="33"/>
-      <c r="L135" s="33"/>
+      <c r="J135" s="34"/>
+      <c r="K135" s="34"/>
+      <c r="L135" s="34"/>
     </row>
     <row r="136" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J136" s="33"/>
-      <c r="K136" s="33"/>
-      <c r="L136" s="33"/>
+      <c r="J136" s="34"/>
+      <c r="K136" s="34"/>
+      <c r="L136" s="34"/>
     </row>
     <row r="137" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J137" s="33"/>
-      <c r="K137" s="33"/>
-      <c r="L137" s="33"/>
+      <c r="J137" s="34"/>
+      <c r="K137" s="34"/>
+      <c r="L137" s="34"/>
     </row>
     <row r="138" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J138" s="33"/>
-      <c r="K138" s="33"/>
-      <c r="L138" s="33"/>
+      <c r="J138" s="34"/>
+      <c r="K138" s="34"/>
+      <c r="L138" s="34"/>
     </row>
     <row r="139" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J139" s="33"/>
-      <c r="K139" s="33"/>
-      <c r="L139" s="33"/>
+      <c r="J139" s="34"/>
+      <c r="K139" s="34"/>
+      <c r="L139" s="34"/>
     </row>
     <row r="140" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J140" s="33"/>
-      <c r="K140" s="33"/>
-      <c r="L140" s="33"/>
+      <c r="J140" s="34"/>
+      <c r="K140" s="34"/>
+      <c r="L140" s="34"/>
     </row>
     <row r="141" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J141" s="33"/>
-      <c r="K141" s="33"/>
-      <c r="L141" s="33"/>
+      <c r="J141" s="34"/>
+      <c r="K141" s="34"/>
+      <c r="L141" s="34"/>
     </row>
     <row r="142" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J142" s="33"/>
-      <c r="K142" s="33"/>
-      <c r="L142" s="33"/>
+      <c r="J142" s="34"/>
+      <c r="K142" s="34"/>
+      <c r="L142" s="34"/>
     </row>
     <row r="143" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J143" s="33"/>
-      <c r="K143" s="33"/>
-      <c r="L143" s="33"/>
+      <c r="J143" s="34"/>
+      <c r="K143" s="34"/>
+      <c r="L143" s="34"/>
     </row>
     <row r="144" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J144" s="33"/>
-      <c r="K144" s="33"/>
-      <c r="L144" s="33"/>
+      <c r="J144" s="34"/>
+      <c r="K144" s="34"/>
+      <c r="L144" s="34"/>
     </row>
     <row r="145" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J145" s="33"/>
-      <c r="K145" s="33"/>
-      <c r="L145" s="33"/>
+      <c r="J145" s="34"/>
+      <c r="K145" s="34"/>
+      <c r="L145" s="34"/>
     </row>
     <row r="146" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J146" s="33"/>
-      <c r="K146" s="33"/>
-      <c r="L146" s="33"/>
+      <c r="J146" s="34"/>
+      <c r="K146" s="34"/>
+      <c r="L146" s="34"/>
     </row>
     <row r="147" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J147" s="33"/>
-      <c r="K147" s="33"/>
-      <c r="L147" s="33"/>
+      <c r="J147" s="34"/>
+      <c r="K147" s="34"/>
+      <c r="L147" s="34"/>
     </row>
     <row r="148" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J148" s="33"/>
-      <c r="K148" s="33"/>
-      <c r="L148" s="33"/>
+      <c r="J148" s="34"/>
+      <c r="K148" s="34"/>
+      <c r="L148" s="34"/>
     </row>
     <row r="149" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J149" s="33"/>
-      <c r="K149" s="33"/>
-      <c r="L149" s="33"/>
+      <c r="J149" s="34"/>
+      <c r="K149" s="34"/>
+      <c r="L149" s="34"/>
     </row>
     <row r="150" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J150" s="33"/>
-      <c r="K150" s="33"/>
-      <c r="L150" s="33"/>
+      <c r="J150" s="34"/>
+      <c r="K150" s="34"/>
+      <c r="L150" s="34"/>
     </row>
     <row r="151" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J151" s="33"/>
-      <c r="K151" s="33"/>
-      <c r="L151" s="33"/>
+      <c r="J151" s="34"/>
+      <c r="K151" s="34"/>
+      <c r="L151" s="34"/>
     </row>
     <row r="152" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J152" s="33"/>
-      <c r="K152" s="33"/>
-      <c r="L152" s="33"/>
+      <c r="J152" s="34"/>
+      <c r="K152" s="34"/>
+      <c r="L152" s="34"/>
     </row>
     <row r="153" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J153" s="33"/>
-      <c r="K153" s="33"/>
-      <c r="L153" s="33"/>
+      <c r="J153" s="34"/>
+      <c r="K153" s="34"/>
+      <c r="L153" s="34"/>
     </row>
     <row r="154" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J154" s="33"/>
-      <c r="K154" s="33"/>
-      <c r="L154" s="33"/>
+      <c r="J154" s="34"/>
+      <c r="K154" s="34"/>
+      <c r="L154" s="34"/>
     </row>
     <row r="155" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J155" s="33"/>
-      <c r="K155" s="33"/>
-      <c r="L155" s="33"/>
+      <c r="J155" s="34"/>
+      <c r="K155" s="34"/>
+      <c r="L155" s="34"/>
     </row>
     <row r="156" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J156" s="33"/>
-      <c r="K156" s="33"/>
-      <c r="L156" s="33"/>
+      <c r="J156" s="34"/>
+      <c r="K156" s="34"/>
+      <c r="L156" s="34"/>
     </row>
     <row r="157" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J157" s="33"/>
-      <c r="K157" s="33"/>
-      <c r="L157" s="33"/>
+      <c r="J157" s="34"/>
+      <c r="K157" s="34"/>
+      <c r="L157" s="34"/>
     </row>
     <row r="158" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J158" s="33"/>
-      <c r="K158" s="33"/>
-      <c r="L158" s="33"/>
+      <c r="J158" s="34"/>
+      <c r="K158" s="34"/>
+      <c r="L158" s="34"/>
     </row>
     <row r="159" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J159" s="33"/>
-      <c r="K159" s="33"/>
-      <c r="L159" s="33"/>
+      <c r="J159" s="34"/>
+      <c r="K159" s="34"/>
+      <c r="L159" s="34"/>
     </row>
     <row r="160" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J160" s="33"/>
-      <c r="K160" s="33"/>
-      <c r="L160" s="33"/>
+      <c r="J160" s="34"/>
+      <c r="K160" s="34"/>
+      <c r="L160" s="34"/>
     </row>
     <row r="161" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J161" s="33"/>
-      <c r="K161" s="33"/>
-      <c r="L161" s="33"/>
+      <c r="J161" s="34"/>
+      <c r="K161" s="34"/>
+      <c r="L161" s="34"/>
     </row>
     <row r="162" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J162" s="33"/>
-      <c r="K162" s="33"/>
-      <c r="L162" s="33"/>
+      <c r="J162" s="34"/>
+      <c r="K162" s="34"/>
+      <c r="L162" s="34"/>
     </row>
     <row r="163" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J163" s="33"/>
-      <c r="K163" s="33"/>
-      <c r="L163" s="33"/>
+      <c r="J163" s="34"/>
+      <c r="K163" s="34"/>
+      <c r="L163" s="34"/>
     </row>
     <row r="164" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J164" s="33"/>
-      <c r="K164" s="33"/>
-      <c r="L164" s="33"/>
+      <c r="J164" s="34"/>
+      <c r="K164" s="34"/>
+      <c r="L164" s="34"/>
     </row>
     <row r="165" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J165" s="33"/>
-      <c r="K165" s="33"/>
-      <c r="L165" s="33"/>
+      <c r="J165" s="34"/>
+      <c r="K165" s="34"/>
+      <c r="L165" s="34"/>
     </row>
     <row r="166" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J166" s="33"/>
-      <c r="K166" s="33"/>
-      <c r="L166" s="33"/>
+      <c r="J166" s="34"/>
+      <c r="K166" s="34"/>
+      <c r="L166" s="34"/>
     </row>
     <row r="167" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J167" s="33"/>
-      <c r="K167" s="33"/>
-      <c r="L167" s="33"/>
+      <c r="J167" s="34"/>
+      <c r="K167" s="34"/>
+      <c r="L167" s="34"/>
     </row>
     <row r="168" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J168" s="33"/>
-      <c r="K168" s="33"/>
-      <c r="L168" s="33"/>
+      <c r="J168" s="34"/>
+      <c r="K168" s="34"/>
+      <c r="L168" s="34"/>
     </row>
     <row r="169" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J169" s="33"/>
-      <c r="K169" s="33"/>
-      <c r="L169" s="33"/>
+      <c r="J169" s="34"/>
+      <c r="K169" s="34"/>
+      <c r="L169" s="34"/>
     </row>
     <row r="170" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J170" s="33"/>
-      <c r="K170" s="33"/>
-      <c r="L170" s="33"/>
+      <c r="J170" s="34"/>
+      <c r="K170" s="34"/>
+      <c r="L170" s="34"/>
     </row>
     <row r="171" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J171" s="33"/>
-      <c r="K171" s="33"/>
-      <c r="L171" s="33"/>
+      <c r="J171" s="34"/>
+      <c r="K171" s="34"/>
+      <c r="L171" s="34"/>
     </row>
     <row r="172" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J172" s="33"/>
-      <c r="K172" s="33"/>
-      <c r="L172" s="33"/>
+      <c r="J172" s="34"/>
+      <c r="K172" s="34"/>
+      <c r="L172" s="34"/>
     </row>
     <row r="173" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J173" s="33"/>
-      <c r="K173" s="33"/>
-      <c r="L173" s="33"/>
+      <c r="J173" s="34"/>
+      <c r="K173" s="34"/>
+      <c r="L173" s="34"/>
     </row>
     <row r="174" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J174" s="33"/>
-      <c r="K174" s="33"/>
-      <c r="L174" s="33"/>
+      <c r="J174" s="34"/>
+      <c r="K174" s="34"/>
+      <c r="L174" s="34"/>
     </row>
     <row r="175" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J175" s="33"/>
-      <c r="K175" s="33"/>
-      <c r="L175" s="33"/>
+      <c r="J175" s="34"/>
+      <c r="K175" s="34"/>
+      <c r="L175" s="34"/>
     </row>
     <row r="176" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J176" s="33"/>
-      <c r="K176" s="33"/>
-      <c r="L176" s="33"/>
+      <c r="J176" s="34"/>
+      <c r="K176" s="34"/>
+      <c r="L176" s="34"/>
     </row>
     <row r="177" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J177" s="33"/>
-      <c r="K177" s="33"/>
-      <c r="L177" s="33"/>
+      <c r="J177" s="34"/>
+      <c r="K177" s="34"/>
+      <c r="L177" s="34"/>
     </row>
     <row r="178" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J178" s="33"/>
-      <c r="K178" s="33"/>
-      <c r="L178" s="33"/>
+      <c r="J178" s="34"/>
+      <c r="K178" s="34"/>
+      <c r="L178" s="34"/>
     </row>
     <row r="179" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J179" s="33"/>
-      <c r="K179" s="33"/>
-      <c r="L179" s="33"/>
+      <c r="J179" s="34"/>
+      <c r="K179" s="34"/>
+      <c r="L179" s="34"/>
     </row>
     <row r="180" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J180" s="33"/>
-      <c r="K180" s="33"/>
-      <c r="L180" s="33"/>
+      <c r="J180" s="34"/>
+      <c r="K180" s="34"/>
+      <c r="L180" s="34"/>
     </row>
     <row r="181" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J181" s="33"/>
-      <c r="K181" s="33"/>
-      <c r="L181" s="33"/>
+      <c r="J181" s="34"/>
+      <c r="K181" s="34"/>
+      <c r="L181" s="34"/>
     </row>
     <row r="182" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J182" s="33"/>
-      <c r="K182" s="33"/>
-      <c r="L182" s="33"/>
+      <c r="J182" s="34"/>
+      <c r="K182" s="34"/>
+      <c r="L182" s="34"/>
     </row>
     <row r="183" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J183" s="33"/>
-      <c r="K183" s="33"/>
-      <c r="L183" s="33"/>
+      <c r="J183" s="34"/>
+      <c r="K183" s="34"/>
+      <c r="L183" s="34"/>
     </row>
     <row r="184" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J184" s="33"/>
-      <c r="K184" s="33"/>
-      <c r="L184" s="33"/>
+      <c r="J184" s="34"/>
+      <c r="K184" s="34"/>
+      <c r="L184" s="34"/>
     </row>
     <row r="185" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J185" s="33"/>
-      <c r="K185" s="33"/>
-      <c r="L185" s="33"/>
+      <c r="J185" s="34"/>
+      <c r="K185" s="34"/>
+      <c r="L185" s="34"/>
     </row>
     <row r="186" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J186" s="33"/>
-      <c r="K186" s="33"/>
-      <c r="L186" s="33"/>
+      <c r="J186" s="34"/>
+      <c r="K186" s="34"/>
+      <c r="L186" s="34"/>
     </row>
     <row r="187" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J187" s="33"/>
-      <c r="K187" s="33"/>
-      <c r="L187" s="33"/>
+      <c r="J187" s="34"/>
+      <c r="K187" s="34"/>
+      <c r="L187" s="34"/>
     </row>
     <row r="188" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J188" s="33"/>
-      <c r="K188" s="33"/>
-      <c r="L188" s="33"/>
+      <c r="J188" s="34"/>
+      <c r="K188" s="34"/>
+      <c r="L188" s="34"/>
     </row>
     <row r="189" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J189" s="33"/>
-      <c r="K189" s="33"/>
-      <c r="L189" s="33"/>
+      <c r="J189" s="34"/>
+      <c r="K189" s="34"/>
+      <c r="L189" s="34"/>
     </row>
     <row r="190" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J190" s="33"/>
-      <c r="K190" s="33"/>
-      <c r="L190" s="33"/>
+      <c r="J190" s="34"/>
+      <c r="K190" s="34"/>
+      <c r="L190" s="34"/>
     </row>
     <row r="191" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J191" s="33"/>
-      <c r="K191" s="33"/>
-      <c r="L191" s="33"/>
+      <c r="J191" s="34"/>
+      <c r="K191" s="34"/>
+      <c r="L191" s="34"/>
     </row>
     <row r="192" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J192" s="33"/>
-      <c r="K192" s="33"/>
-      <c r="L192" s="33"/>
+      <c r="J192" s="34"/>
+      <c r="K192" s="34"/>
+      <c r="L192" s="34"/>
     </row>
     <row r="193" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J193" s="33"/>
-      <c r="K193" s="33"/>
-      <c r="L193" s="33"/>
+      <c r="J193" s="34"/>
+      <c r="K193" s="34"/>
+      <c r="L193" s="34"/>
     </row>
     <row r="194" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J194" s="33"/>
-      <c r="K194" s="33"/>
-      <c r="L194" s="33"/>
+      <c r="J194" s="34"/>
+      <c r="K194" s="34"/>
+      <c r="L194" s="34"/>
     </row>
     <row r="195" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J195" s="33"/>
-      <c r="K195" s="33"/>
-      <c r="L195" s="33"/>
+      <c r="J195" s="34"/>
+      <c r="K195" s="34"/>
+      <c r="L195" s="34"/>
     </row>
     <row r="196" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J196" s="33"/>
-      <c r="K196" s="33"/>
-      <c r="L196" s="33"/>
+      <c r="J196" s="34"/>
+      <c r="K196" s="34"/>
+      <c r="L196" s="34"/>
     </row>
     <row r="197" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J197" s="33"/>
-      <c r="K197" s="33"/>
-      <c r="L197" s="33"/>
+      <c r="J197" s="34"/>
+      <c r="K197" s="34"/>
+      <c r="L197" s="34"/>
     </row>
     <row r="198" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J198" s="33"/>
-      <c r="K198" s="33"/>
-      <c r="L198" s="33"/>
+      <c r="J198" s="34"/>
+      <c r="K198" s="34"/>
+      <c r="L198" s="34"/>
     </row>
     <row r="199" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J199" s="33"/>
-      <c r="K199" s="33"/>
-      <c r="L199" s="33"/>
+      <c r="J199" s="34"/>
+      <c r="K199" s="34"/>
+      <c r="L199" s="34"/>
     </row>
     <row r="200" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J200" s="33"/>
-      <c r="K200" s="33"/>
-      <c r="L200" s="33"/>
+      <c r="J200" s="34"/>
+      <c r="K200" s="34"/>
+      <c r="L200" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
chore: update test data file for improved test coverage and accuracy
</commit_message>
<xml_diff>
--- a/test_data/data.xlsx
+++ b/test_data/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Linh\Đồ án\DATN\linky-testing\test_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{125EE1DE-CD48-4F8B-904C-1D9ABB76B920}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C103700-54E2-4552-ACFE-A78750B0C076}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="95">
   <si>
     <t>email</t>
   </si>
@@ -299,6 +299,18 @@
   </si>
   <si>
     <t>Hà Nội</t>
+  </si>
+  <si>
+    <t>section</t>
+  </si>
+  <si>
+    <t>profile-header</t>
+  </si>
+  <si>
+    <t>personal</t>
+  </si>
+  <si>
+    <t>interests</t>
   </si>
 </sst>
 </file>
@@ -341,7 +353,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -353,8 +365,14 @@
         <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -479,12 +497,36 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFC6C6C6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -580,21 +622,29 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1380,538 +1430,625 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.1640625" style="20" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" style="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.75" style="20" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.1640625" style="20" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.4140625" style="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.75" style="20" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.1640625" style="20" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.1640625" style="20" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.58203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.1640625" style="20" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" style="20" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.75" style="20" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.1640625" style="20" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.4140625" style="21" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.75" style="20" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.1640625" style="20" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.1640625" style="20" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.58203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="40" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="C1" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="D1" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="E1" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="F1" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="G1" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="16"/>
-      <c r="B2" s="16"/>
+    <row r="2" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="34"/>
       <c r="C2" s="16"/>
-      <c r="D2" s="16" t="s">
+      <c r="D2" s="16"/>
+      <c r="E2" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="E2" s="17"/>
-      <c r="F2" s="16"/>
+      <c r="F2" s="17"/>
       <c r="G2" s="16"/>
-      <c r="H2" s="16" t="s">
+      <c r="H2" s="16"/>
+      <c r="I2" s="16" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="16"/>
+    <row r="3" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="41" t="s">
+        <v>28</v>
+      </c>
       <c r="B3" s="16"/>
       <c r="C3" s="16"/>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="16"/>
+      <c r="E3" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="17"/>
-      <c r="F3" s="16"/>
+      <c r="F3" s="17"/>
       <c r="G3" s="16"/>
-      <c r="H3" s="16" t="s">
+      <c r="H3" s="16"/>
+      <c r="I3" s="16" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="16"/>
+    <row r="4" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="41" t="s">
+        <v>28</v>
+      </c>
       <c r="B4" s="16"/>
       <c r="C4" s="16"/>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="16"/>
+      <c r="E4" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E4" s="17"/>
-      <c r="F4" s="16"/>
+      <c r="F4" s="17"/>
       <c r="G4" s="16"/>
-      <c r="H4" s="16" t="s">
+      <c r="H4" s="16"/>
+      <c r="I4" s="16" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="16"/>
+    <row r="5" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="41" t="s">
+        <v>28</v>
+      </c>
       <c r="B5" s="16"/>
       <c r="C5" s="16"/>
-      <c r="D5" s="16" t="s">
+      <c r="D5" s="16"/>
+      <c r="E5" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="E5" s="17"/>
-      <c r="F5" s="16"/>
+      <c r="F5" s="17"/>
       <c r="G5" s="16"/>
-      <c r="H5" s="16" t="s">
+      <c r="H5" s="16"/>
+      <c r="I5" s="16" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="16"/>
+    <row r="6" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="41" t="s">
+        <v>28</v>
+      </c>
       <c r="B6" s="16"/>
       <c r="C6" s="16"/>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="16"/>
+      <c r="E6" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="E6" s="17"/>
-      <c r="F6" s="16"/>
+      <c r="F6" s="17"/>
       <c r="G6" s="16"/>
-      <c r="H6" s="16" t="s">
+      <c r="H6" s="16"/>
+      <c r="I6" s="16" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="16"/>
+    <row r="7" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="41" t="s">
+        <v>28</v>
+      </c>
       <c r="B7" s="16"/>
       <c r="C7" s="16"/>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="16"/>
+      <c r="E7" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="E7" s="17"/>
-      <c r="F7" s="16"/>
+      <c r="F7" s="17"/>
       <c r="G7" s="16"/>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="16"/>
+      <c r="I7" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="I7" s="19"/>
-    </row>
-    <row r="8" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="16" t="s">
+      <c r="J7" s="19"/>
+    </row>
+    <row r="8" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="42" t="s">
+        <v>92</v>
+      </c>
+      <c r="B8" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="16"/>
       <c r="C8" s="16"/>
       <c r="D8" s="16"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="17"/>
       <c r="G8" s="16"/>
-      <c r="H8" s="16" t="s">
+      <c r="H8" s="16"/>
+      <c r="I8" s="16" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="16"/>
-      <c r="B9" s="16" t="s">
+    <row r="9" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="42" t="s">
+        <v>92</v>
+      </c>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="16"/>
       <c r="D9" s="16"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="17"/>
       <c r="G9" s="16"/>
-      <c r="H9" s="9" t="s">
+      <c r="H9" s="16"/>
+      <c r="I9" s="9" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="16" t="s">
+    <row r="10" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="42" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="16" t="s">
+      <c r="C10" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="16"/>
       <c r="D10" s="16"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="17"/>
       <c r="G10" s="16"/>
-      <c r="H10" s="16" t="s">
+      <c r="H10" s="16"/>
+      <c r="I10" s="16" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="16"/>
+    <row r="11" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="42" t="s">
+        <v>92</v>
+      </c>
       <c r="B11" s="16"/>
       <c r="C11" s="16"/>
       <c r="D11" s="16"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="17"/>
       <c r="G11" s="16"/>
-      <c r="H11" s="9" t="s">
+      <c r="H11" s="16"/>
+      <c r="I11" s="9" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="16"/>
+    <row r="12" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="42" t="s">
+        <v>92</v>
+      </c>
       <c r="B12" s="16"/>
-      <c r="C12" s="19" t="s">
+      <c r="C12" s="16"/>
+      <c r="D12" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="D12" s="16"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="17"/>
       <c r="G12" s="16"/>
-      <c r="H12" s="16" t="s">
+      <c r="H12" s="16"/>
+      <c r="I12" s="16" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="16"/>
-      <c r="B13" s="35"/>
-      <c r="C13" s="38" t="s">
+    <row r="13" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="42" t="s">
+        <v>92</v>
+      </c>
+      <c r="B13" s="16"/>
+      <c r="C13" s="33"/>
+      <c r="D13" s="36" t="s">
         <v>90</v>
       </c>
-      <c r="D13" s="36"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="16"/>
+      <c r="E13" s="34"/>
+      <c r="F13" s="17"/>
       <c r="G13" s="16"/>
-      <c r="H13" s="16" t="s">
+      <c r="H13" s="16"/>
+      <c r="I13" s="16" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="16"/>
+    <row r="14" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="42" t="s">
+        <v>92</v>
+      </c>
       <c r="B14" s="16"/>
-      <c r="C14" s="37" t="s">
+      <c r="C14" s="16"/>
+      <c r="D14" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="D14" s="16"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="17"/>
       <c r="G14" s="16"/>
-      <c r="H14" s="16" t="s">
+      <c r="H14" s="16"/>
+      <c r="I14" s="16" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="16" t="s">
+    <row r="15" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="42" t="s">
+        <v>92</v>
+      </c>
+      <c r="B15" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="B15" s="16" t="s">
+      <c r="C15" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="D15" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="D15" s="16"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="17"/>
       <c r="G15" s="16"/>
-      <c r="H15" s="16" t="s">
+      <c r="H15" s="16"/>
+      <c r="I15" s="16" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="16" t="s">
+    <row r="16" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="42" t="s">
+        <v>92</v>
+      </c>
+      <c r="B16" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="B16" s="16" t="s">
+      <c r="C16" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="C16" s="16"/>
       <c r="D16" s="16"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="17"/>
       <c r="G16" s="16"/>
-      <c r="H16" s="9" t="s">
+      <c r="H16" s="16"/>
+      <c r="I16" s="9" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="9" t="s">
+    <row r="17" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="42" t="s">
+        <v>92</v>
+      </c>
+      <c r="B17" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="B17" s="16"/>
       <c r="C17" s="16"/>
       <c r="D17" s="16"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="17"/>
       <c r="G17" s="16"/>
-      <c r="H17" s="9" t="s">
+      <c r="H17" s="16"/>
+      <c r="I17" s="9" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="9" t="s">
+    <row r="18" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="42" t="s">
+        <v>92</v>
+      </c>
+      <c r="B18" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="B18" s="16"/>
       <c r="C18" s="16"/>
       <c r="D18" s="16"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="17"/>
       <c r="G18" s="16"/>
-      <c r="H18" s="16" t="s">
+      <c r="H18" s="16"/>
+      <c r="I18" s="16" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="9" t="s">
+    <row r="19" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="42" t="s">
+        <v>92</v>
+      </c>
+      <c r="B19" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="B19" s="16"/>
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="16"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="17"/>
       <c r="G19" s="16"/>
-      <c r="H19" s="9" t="s">
+      <c r="H19" s="16"/>
+      <c r="I19" s="9" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="16"/>
+    <row r="20" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="42" t="s">
+        <v>93</v>
+      </c>
       <c r="B20" s="16"/>
       <c r="C20" s="16"/>
       <c r="D20" s="16"/>
-      <c r="E20" s="17" t="s">
+      <c r="E20" s="16"/>
+      <c r="F20" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="F20" s="16"/>
       <c r="G20" s="16"/>
-      <c r="H20" s="9" t="s">
+      <c r="H20" s="16"/>
+      <c r="I20" s="9" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="16"/>
+    <row r="21" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="42" t="s">
+        <v>93</v>
+      </c>
       <c r="B21" s="16"/>
       <c r="C21" s="16"/>
       <c r="D21" s="16"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="16" t="s">
+      <c r="E21" s="16"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="G21" s="16"/>
-      <c r="H21" s="9" t="s">
+      <c r="H21" s="16"/>
+      <c r="I21" s="9" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="16"/>
+    <row r="22" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="42" t="s">
+        <v>93</v>
+      </c>
       <c r="B22" s="16"/>
       <c r="C22" s="16"/>
       <c r="D22" s="16"/>
-      <c r="E22" s="17">
+      <c r="E22" s="16"/>
+      <c r="F22" s="17">
         <v>37956</v>
       </c>
-      <c r="F22" s="19" t="s">
+      <c r="G22" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="G22" s="16"/>
-      <c r="H22" s="9" t="s">
+      <c r="H22" s="16"/>
+      <c r="I22" s="9" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="16"/>
+    <row r="23" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="42" t="s">
+        <v>93</v>
+      </c>
       <c r="B23" s="16"/>
       <c r="C23" s="16"/>
       <c r="D23" s="16"/>
-      <c r="E23" s="17" t="s">
+      <c r="E23" s="16"/>
+      <c r="F23" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="F23" s="16" t="s">
+      <c r="G23" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="G23" s="16"/>
-      <c r="H23" s="9" t="s">
+      <c r="H23" s="16"/>
+      <c r="I23" s="9" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="16"/>
+    <row r="24" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="42" t="s">
+        <v>93</v>
+      </c>
       <c r="B24" s="16"/>
       <c r="C24" s="16"/>
       <c r="D24" s="16"/>
-      <c r="E24" s="17" t="s">
+      <c r="E24" s="16"/>
+      <c r="F24" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="F24" s="16"/>
       <c r="G24" s="16"/>
-      <c r="H24" s="9" t="s">
+      <c r="H24" s="16"/>
+      <c r="I24" s="9" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="16"/>
+    <row r="25" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="42" t="s">
+        <v>93</v>
+      </c>
       <c r="B25" s="16"/>
       <c r="C25" s="16"/>
       <c r="D25" s="16"/>
-      <c r="E25" s="17">
+      <c r="E25" s="16"/>
+      <c r="F25" s="17">
         <v>36526</v>
       </c>
-      <c r="F25" s="16"/>
       <c r="G25" s="16"/>
-      <c r="H25" s="9" t="s">
+      <c r="H25" s="16"/>
+      <c r="I25" s="9" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="16"/>
+    <row r="26" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="42" t="s">
+        <v>94</v>
+      </c>
       <c r="B26" s="16"/>
       <c r="C26" s="16"/>
       <c r="D26" s="16"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="16"/>
-      <c r="G26" s="16" t="s">
+      <c r="E26" s="16"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="16"/>
+      <c r="H26" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="H26" s="16" t="s">
+      <c r="I26" s="16" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="16"/>
+    <row r="27" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="42" t="s">
+        <v>94</v>
+      </c>
       <c r="B27" s="16"/>
       <c r="C27" s="16"/>
       <c r="D27" s="16"/>
-      <c r="E27" s="17"/>
-      <c r="F27" s="16"/>
-      <c r="G27" s="16" t="s">
+      <c r="E27" s="16"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="16"/>
+      <c r="H27" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="H27" s="16" t="s">
+      <c r="I27" s="16" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="16"/>
+    <row r="28" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="42" t="s">
+        <v>94</v>
+      </c>
       <c r="B28" s="16"/>
       <c r="C28" s="16"/>
       <c r="D28" s="16"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="16" t="s">
+      <c r="E28" s="16"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="16"/>
+      <c r="H28" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="H28" s="16" t="s">
+      <c r="I28" s="16" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="16"/>
+    <row r="29" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="42" t="s">
+        <v>94</v>
+      </c>
       <c r="B29" s="16"/>
       <c r="C29" s="16"/>
       <c r="D29" s="16"/>
-      <c r="E29" s="17"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="16" t="s">
+      <c r="E29" s="16"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="16"/>
+      <c r="H29" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="H29" s="7" t="s">
+      <c r="I29" s="7" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="16"/>
+    <row r="30" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B30" s="16"/>
       <c r="C30" s="16"/>
       <c r="D30" s="16"/>
-      <c r="E30" s="17"/>
-      <c r="F30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="17"/>
       <c r="G30" s="16"/>
       <c r="H30" s="16"/>
-    </row>
-    <row r="31" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="16"/>
+      <c r="I30" s="16"/>
+    </row>
+    <row r="31" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B31" s="16"/>
       <c r="C31" s="16"/>
       <c r="D31" s="16"/>
-      <c r="E31" s="17"/>
-      <c r="F31" s="16"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="17"/>
       <c r="G31" s="16"/>
       <c r="H31" s="16"/>
-    </row>
-    <row r="32" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="16"/>
+      <c r="I31" s="16"/>
+    </row>
+    <row r="32" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B32" s="16"/>
       <c r="C32" s="16"/>
       <c r="D32" s="16"/>
-      <c r="E32" s="17"/>
-      <c r="F32" s="16"/>
+      <c r="E32" s="16"/>
+      <c r="F32" s="17"/>
       <c r="G32" s="16"/>
       <c r="H32" s="16"/>
-    </row>
-    <row r="33" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="16"/>
+      <c r="I32" s="16"/>
+    </row>
+    <row r="33" spans="2:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B33" s="16"/>
       <c r="C33" s="16"/>
       <c r="D33" s="16"/>
-      <c r="E33" s="17"/>
-      <c r="F33" s="16"/>
+      <c r="E33" s="16"/>
+      <c r="F33" s="17"/>
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
-    </row>
-    <row r="34" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="16"/>
+      <c r="I33" s="16"/>
+    </row>
+    <row r="34" spans="2:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B34" s="16"/>
       <c r="C34" s="16"/>
       <c r="D34" s="16"/>
-      <c r="E34" s="17"/>
-      <c r="F34" s="16"/>
+      <c r="E34" s="16"/>
+      <c r="F34" s="17"/>
       <c r="G34" s="16"/>
       <c r="H34" s="16"/>
-    </row>
-    <row r="35" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="16"/>
+      <c r="I34" s="16"/>
+    </row>
+    <row r="35" spans="2:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B35" s="16"/>
       <c r="C35" s="16"/>
       <c r="D35" s="16"/>
-      <c r="E35" s="17"/>
-      <c r="F35" s="16"/>
+      <c r="E35" s="16"/>
+      <c r="F35" s="17"/>
       <c r="G35" s="16"/>
       <c r="H35" s="16"/>
-    </row>
-    <row r="36" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="16"/>
+      <c r="I35" s="16"/>
+    </row>
+    <row r="36" spans="2:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B36" s="16"/>
       <c r="C36" s="16"/>
       <c r="D36" s="16"/>
-      <c r="E36" s="17"/>
-      <c r="F36" s="16"/>
+      <c r="E36" s="16"/>
+      <c r="F36" s="17"/>
       <c r="G36" s="16"/>
       <c r="H36" s="16"/>
-    </row>
-    <row r="37" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="16"/>
+      <c r="I36" s="16"/>
+    </row>
+    <row r="37" spans="2:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B37" s="16"/>
       <c r="C37" s="16"/>
       <c r="D37" s="16"/>
-      <c r="E37" s="17"/>
-      <c r="F37" s="16"/>
+      <c r="E37" s="16"/>
+      <c r="F37" s="17"/>
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
-    </row>
-    <row r="38" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="16"/>
+      <c r="I37" s="16"/>
+    </row>
+    <row r="38" spans="2:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B38" s="16"/>
       <c r="C38" s="16"/>
       <c r="D38" s="16"/>
-      <c r="E38" s="17"/>
-      <c r="F38" s="16"/>
+      <c r="E38" s="16"/>
+      <c r="F38" s="17"/>
       <c r="G38" s="16"/>
       <c r="H38" s="16"/>
+      <c r="I38" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1961,9 +2098,9 @@
       </c>
       <c r="H1" s="4"/>
       <c r="I1" s="4"/>
-      <c r="J1" s="33"/>
-      <c r="K1" s="34"/>
-      <c r="L1" s="34"/>
+      <c r="J1" s="37"/>
+      <c r="K1" s="38"/>
+      <c r="L1" s="38"/>
       <c r="M1" s="4"/>
       <c r="N1" s="4"/>
       <c r="O1" s="4"/>
@@ -2178,9 +2315,9 @@
       <c r="G2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="34"/>
-      <c r="K2" s="34"/>
-      <c r="L2" s="34"/>
+      <c r="J2" s="38"/>
+      <c r="K2" s="38"/>
+      <c r="L2" s="38"/>
     </row>
     <row r="3" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
@@ -2198,9 +2335,9 @@
       <c r="G3" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="34"/>
-      <c r="K3" s="34"/>
-      <c r="L3" s="34"/>
+      <c r="J3" s="38"/>
+      <c r="K3" s="38"/>
+      <c r="L3" s="38"/>
     </row>
     <row r="4" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
@@ -2224,9 +2361,9 @@
       <c r="G4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="J4" s="34"/>
-      <c r="K4" s="34"/>
-      <c r="L4" s="34"/>
+      <c r="J4" s="38"/>
+      <c r="K4" s="38"/>
+      <c r="L4" s="38"/>
     </row>
     <row r="5" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
@@ -2250,9 +2387,9 @@
       <c r="G5" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="J5" s="34"/>
-      <c r="K5" s="34"/>
-      <c r="L5" s="34"/>
+      <c r="J5" s="38"/>
+      <c r="K5" s="38"/>
+      <c r="L5" s="38"/>
     </row>
     <row r="6" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
@@ -2276,9 +2413,9 @@
       <c r="G6" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="J6" s="34"/>
-      <c r="K6" s="34"/>
-      <c r="L6" s="34"/>
+      <c r="J6" s="38"/>
+      <c r="K6" s="38"/>
+      <c r="L6" s="38"/>
     </row>
     <row r="7" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
@@ -2302,9 +2439,9 @@
       <c r="G7" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="J7" s="34"/>
-      <c r="K7" s="34"/>
-      <c r="L7" s="34"/>
+      <c r="J7" s="38"/>
+      <c r="K7" s="38"/>
+      <c r="L7" s="38"/>
     </row>
     <row r="8" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
@@ -2328,9 +2465,9 @@
       <c r="G8" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="J8" s="34"/>
-      <c r="K8" s="34"/>
-      <c r="L8" s="34"/>
+      <c r="J8" s="38"/>
+      <c r="K8" s="38"/>
+      <c r="L8" s="38"/>
     </row>
     <row r="9" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
@@ -2354,9 +2491,9 @@
       <c r="G9" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="J9" s="34"/>
-      <c r="K9" s="34"/>
-      <c r="L9" s="34"/>
+      <c r="J9" s="38"/>
+      <c r="K9" s="38"/>
+      <c r="L9" s="38"/>
     </row>
     <row r="10" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
@@ -2380,9 +2517,9 @@
       <c r="G10" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="J10" s="34"/>
-      <c r="K10" s="34"/>
-      <c r="L10" s="34"/>
+      <c r="J10" s="38"/>
+      <c r="K10" s="38"/>
+      <c r="L10" s="38"/>
     </row>
     <row r="11" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
@@ -2406,9 +2543,9 @@
       <c r="G11" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="J11" s="34"/>
-      <c r="K11" s="34"/>
-      <c r="L11" s="34"/>
+      <c r="J11" s="38"/>
+      <c r="K11" s="38"/>
+      <c r="L11" s="38"/>
     </row>
     <row r="12" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
@@ -2432,9 +2569,9 @@
       <c r="G12" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="J12" s="34"/>
-      <c r="K12" s="34"/>
-      <c r="L12" s="34"/>
+      <c r="J12" s="38"/>
+      <c r="K12" s="38"/>
+      <c r="L12" s="38"/>
     </row>
     <row r="13" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
@@ -2458,9 +2595,9 @@
       <c r="G13" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="J13" s="34"/>
-      <c r="K13" s="34"/>
-      <c r="L13" s="34"/>
+      <c r="J13" s="38"/>
+      <c r="K13" s="38"/>
+      <c r="L13" s="38"/>
     </row>
     <row r="14" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
@@ -2484,9 +2621,9 @@
       <c r="G14" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="J14" s="34"/>
-      <c r="K14" s="34"/>
-      <c r="L14" s="34"/>
+      <c r="J14" s="38"/>
+      <c r="K14" s="38"/>
+      <c r="L14" s="38"/>
     </row>
     <row r="15" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
@@ -2510,9 +2647,9 @@
       <c r="G15" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="J15" s="34"/>
-      <c r="K15" s="34"/>
-      <c r="L15" s="34"/>
+      <c r="J15" s="38"/>
+      <c r="K15" s="38"/>
+      <c r="L15" s="38"/>
     </row>
     <row r="16" spans="1:209" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
@@ -2536,9 +2673,9 @@
       <c r="G16" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="J16" s="34"/>
-      <c r="K16" s="34"/>
-      <c r="L16" s="34"/>
+      <c r="J16" s="38"/>
+      <c r="K16" s="38"/>
+      <c r="L16" s="38"/>
     </row>
     <row r="17" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
@@ -2562,9 +2699,9 @@
       <c r="G17" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="J17" s="34"/>
-      <c r="K17" s="34"/>
-      <c r="L17" s="34"/>
+      <c r="J17" s="38"/>
+      <c r="K17" s="38"/>
+      <c r="L17" s="38"/>
     </row>
     <row r="18" spans="1:12" ht="83.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
@@ -2588,919 +2725,919 @@
       <c r="G18" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="J18" s="34"/>
-      <c r="K18" s="34"/>
-      <c r="L18" s="34"/>
+      <c r="J18" s="38"/>
+      <c r="K18" s="38"/>
+      <c r="L18" s="38"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J19" s="34"/>
-      <c r="K19" s="34"/>
-      <c r="L19" s="34"/>
+      <c r="J19" s="38"/>
+      <c r="K19" s="38"/>
+      <c r="L19" s="38"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J20" s="34"/>
-      <c r="K20" s="34"/>
-      <c r="L20" s="34"/>
+      <c r="J20" s="38"/>
+      <c r="K20" s="38"/>
+      <c r="L20" s="38"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J21" s="34"/>
-      <c r="K21" s="34"/>
-      <c r="L21" s="34"/>
+      <c r="J21" s="38"/>
+      <c r="K21" s="38"/>
+      <c r="L21" s="38"/>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J22" s="34"/>
-      <c r="K22" s="34"/>
-      <c r="L22" s="34"/>
+      <c r="J22" s="38"/>
+      <c r="K22" s="38"/>
+      <c r="L22" s="38"/>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J23" s="34"/>
-      <c r="K23" s="34"/>
-      <c r="L23" s="34"/>
+      <c r="J23" s="38"/>
+      <c r="K23" s="38"/>
+      <c r="L23" s="38"/>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J24" s="34"/>
-      <c r="K24" s="34"/>
-      <c r="L24" s="34"/>
+      <c r="J24" s="38"/>
+      <c r="K24" s="38"/>
+      <c r="L24" s="38"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J25" s="34"/>
-      <c r="K25" s="34"/>
-      <c r="L25" s="34"/>
+      <c r="J25" s="38"/>
+      <c r="K25" s="38"/>
+      <c r="L25" s="38"/>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J26" s="34"/>
-      <c r="K26" s="34"/>
-      <c r="L26" s="34"/>
+      <c r="J26" s="38"/>
+      <c r="K26" s="38"/>
+      <c r="L26" s="38"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J27" s="34"/>
-      <c r="K27" s="34"/>
-      <c r="L27" s="34"/>
+      <c r="J27" s="38"/>
+      <c r="K27" s="38"/>
+      <c r="L27" s="38"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J28" s="34"/>
-      <c r="K28" s="34"/>
-      <c r="L28" s="34"/>
+      <c r="J28" s="38"/>
+      <c r="K28" s="38"/>
+      <c r="L28" s="38"/>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J29" s="34"/>
-      <c r="K29" s="34"/>
-      <c r="L29" s="34"/>
+      <c r="J29" s="38"/>
+      <c r="K29" s="38"/>
+      <c r="L29" s="38"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J30" s="34"/>
-      <c r="K30" s="34"/>
-      <c r="L30" s="34"/>
+      <c r="J30" s="38"/>
+      <c r="K30" s="38"/>
+      <c r="L30" s="38"/>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J31" s="34"/>
-      <c r="K31" s="34"/>
-      <c r="L31" s="34"/>
+      <c r="J31" s="38"/>
+      <c r="K31" s="38"/>
+      <c r="L31" s="38"/>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="J32" s="34"/>
-      <c r="K32" s="34"/>
-      <c r="L32" s="34"/>
+      <c r="J32" s="38"/>
+      <c r="K32" s="38"/>
+      <c r="L32" s="38"/>
     </row>
     <row r="33" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J33" s="34"/>
-      <c r="K33" s="34"/>
-      <c r="L33" s="34"/>
+      <c r="J33" s="38"/>
+      <c r="K33" s="38"/>
+      <c r="L33" s="38"/>
     </row>
     <row r="34" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J34" s="34"/>
-      <c r="K34" s="34"/>
-      <c r="L34" s="34"/>
+      <c r="J34" s="38"/>
+      <c r="K34" s="38"/>
+      <c r="L34" s="38"/>
     </row>
     <row r="35" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J35" s="34"/>
-      <c r="K35" s="34"/>
-      <c r="L35" s="34"/>
+      <c r="J35" s="38"/>
+      <c r="K35" s="38"/>
+      <c r="L35" s="38"/>
     </row>
     <row r="36" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J36" s="34"/>
-      <c r="K36" s="34"/>
-      <c r="L36" s="34"/>
+      <c r="J36" s="38"/>
+      <c r="K36" s="38"/>
+      <c r="L36" s="38"/>
     </row>
     <row r="37" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J37" s="34"/>
-      <c r="K37" s="34"/>
-      <c r="L37" s="34"/>
+      <c r="J37" s="38"/>
+      <c r="K37" s="38"/>
+      <c r="L37" s="38"/>
     </row>
     <row r="38" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J38" s="34"/>
-      <c r="K38" s="34"/>
-      <c r="L38" s="34"/>
+      <c r="J38" s="38"/>
+      <c r="K38" s="38"/>
+      <c r="L38" s="38"/>
     </row>
     <row r="39" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J39" s="34"/>
-      <c r="K39" s="34"/>
-      <c r="L39" s="34"/>
+      <c r="J39" s="38"/>
+      <c r="K39" s="38"/>
+      <c r="L39" s="38"/>
     </row>
     <row r="40" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J40" s="34"/>
-      <c r="K40" s="34"/>
-      <c r="L40" s="34"/>
+      <c r="J40" s="38"/>
+      <c r="K40" s="38"/>
+      <c r="L40" s="38"/>
     </row>
     <row r="41" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J41" s="34"/>
-      <c r="K41" s="34"/>
-      <c r="L41" s="34"/>
+      <c r="J41" s="38"/>
+      <c r="K41" s="38"/>
+      <c r="L41" s="38"/>
     </row>
     <row r="42" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J42" s="34"/>
-      <c r="K42" s="34"/>
-      <c r="L42" s="34"/>
+      <c r="J42" s="38"/>
+      <c r="K42" s="38"/>
+      <c r="L42" s="38"/>
     </row>
     <row r="43" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J43" s="34"/>
-      <c r="K43" s="34"/>
-      <c r="L43" s="34"/>
+      <c r="J43" s="38"/>
+      <c r="K43" s="38"/>
+      <c r="L43" s="38"/>
     </row>
     <row r="44" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J44" s="34"/>
-      <c r="K44" s="34"/>
-      <c r="L44" s="34"/>
+      <c r="J44" s="38"/>
+      <c r="K44" s="38"/>
+      <c r="L44" s="38"/>
     </row>
     <row r="45" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J45" s="34"/>
-      <c r="K45" s="34"/>
-      <c r="L45" s="34"/>
+      <c r="J45" s="38"/>
+      <c r="K45" s="38"/>
+      <c r="L45" s="38"/>
     </row>
     <row r="46" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J46" s="34"/>
-      <c r="K46" s="34"/>
-      <c r="L46" s="34"/>
+      <c r="J46" s="38"/>
+      <c r="K46" s="38"/>
+      <c r="L46" s="38"/>
     </row>
     <row r="47" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J47" s="34"/>
-      <c r="K47" s="34"/>
-      <c r="L47" s="34"/>
+      <c r="J47" s="38"/>
+      <c r="K47" s="38"/>
+      <c r="L47" s="38"/>
     </row>
     <row r="48" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J48" s="34"/>
-      <c r="K48" s="34"/>
-      <c r="L48" s="34"/>
+      <c r="J48" s="38"/>
+      <c r="K48" s="38"/>
+      <c r="L48" s="38"/>
     </row>
     <row r="49" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J49" s="34"/>
-      <c r="K49" s="34"/>
-      <c r="L49" s="34"/>
+      <c r="J49" s="38"/>
+      <c r="K49" s="38"/>
+      <c r="L49" s="38"/>
     </row>
     <row r="50" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J50" s="34"/>
-      <c r="K50" s="34"/>
-      <c r="L50" s="34"/>
+      <c r="J50" s="38"/>
+      <c r="K50" s="38"/>
+      <c r="L50" s="38"/>
     </row>
     <row r="51" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J51" s="34"/>
-      <c r="K51" s="34"/>
-      <c r="L51" s="34"/>
+      <c r="J51" s="38"/>
+      <c r="K51" s="38"/>
+      <c r="L51" s="38"/>
     </row>
     <row r="52" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J52" s="34"/>
-      <c r="K52" s="34"/>
-      <c r="L52" s="34"/>
+      <c r="J52" s="38"/>
+      <c r="K52" s="38"/>
+      <c r="L52" s="38"/>
     </row>
     <row r="53" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J53" s="34"/>
-      <c r="K53" s="34"/>
-      <c r="L53" s="34"/>
+      <c r="J53" s="38"/>
+      <c r="K53" s="38"/>
+      <c r="L53" s="38"/>
     </row>
     <row r="54" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J54" s="34"/>
-      <c r="K54" s="34"/>
-      <c r="L54" s="34"/>
+      <c r="J54" s="38"/>
+      <c r="K54" s="38"/>
+      <c r="L54" s="38"/>
     </row>
     <row r="55" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J55" s="34"/>
-      <c r="K55" s="34"/>
-      <c r="L55" s="34"/>
+      <c r="J55" s="38"/>
+      <c r="K55" s="38"/>
+      <c r="L55" s="38"/>
     </row>
     <row r="56" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J56" s="34"/>
-      <c r="K56" s="34"/>
-      <c r="L56" s="34"/>
+      <c r="J56" s="38"/>
+      <c r="K56" s="38"/>
+      <c r="L56" s="38"/>
     </row>
     <row r="57" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J57" s="34"/>
-      <c r="K57" s="34"/>
-      <c r="L57" s="34"/>
+      <c r="J57" s="38"/>
+      <c r="K57" s="38"/>
+      <c r="L57" s="38"/>
     </row>
     <row r="58" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J58" s="34"/>
-      <c r="K58" s="34"/>
-      <c r="L58" s="34"/>
+      <c r="J58" s="38"/>
+      <c r="K58" s="38"/>
+      <c r="L58" s="38"/>
     </row>
     <row r="59" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J59" s="34"/>
-      <c r="K59" s="34"/>
-      <c r="L59" s="34"/>
+      <c r="J59" s="38"/>
+      <c r="K59" s="38"/>
+      <c r="L59" s="38"/>
     </row>
     <row r="60" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J60" s="34"/>
-      <c r="K60" s="34"/>
-      <c r="L60" s="34"/>
+      <c r="J60" s="38"/>
+      <c r="K60" s="38"/>
+      <c r="L60" s="38"/>
     </row>
     <row r="61" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J61" s="34"/>
-      <c r="K61" s="34"/>
-      <c r="L61" s="34"/>
+      <c r="J61" s="38"/>
+      <c r="K61" s="38"/>
+      <c r="L61" s="38"/>
     </row>
     <row r="62" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J62" s="34"/>
-      <c r="K62" s="34"/>
-      <c r="L62" s="34"/>
+      <c r="J62" s="38"/>
+      <c r="K62" s="38"/>
+      <c r="L62" s="38"/>
     </row>
     <row r="63" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J63" s="34"/>
-      <c r="K63" s="34"/>
-      <c r="L63" s="34"/>
+      <c r="J63" s="38"/>
+      <c r="K63" s="38"/>
+      <c r="L63" s="38"/>
     </row>
     <row r="64" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J64" s="34"/>
-      <c r="K64" s="34"/>
-      <c r="L64" s="34"/>
+      <c r="J64" s="38"/>
+      <c r="K64" s="38"/>
+      <c r="L64" s="38"/>
     </row>
     <row r="65" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J65" s="34"/>
-      <c r="K65" s="34"/>
-      <c r="L65" s="34"/>
+      <c r="J65" s="38"/>
+      <c r="K65" s="38"/>
+      <c r="L65" s="38"/>
     </row>
     <row r="66" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J66" s="34"/>
-      <c r="K66" s="34"/>
-      <c r="L66" s="34"/>
+      <c r="J66" s="38"/>
+      <c r="K66" s="38"/>
+      <c r="L66" s="38"/>
     </row>
     <row r="67" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J67" s="34"/>
-      <c r="K67" s="34"/>
-      <c r="L67" s="34"/>
+      <c r="J67" s="38"/>
+      <c r="K67" s="38"/>
+      <c r="L67" s="38"/>
     </row>
     <row r="68" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J68" s="34"/>
-      <c r="K68" s="34"/>
-      <c r="L68" s="34"/>
+      <c r="J68" s="38"/>
+      <c r="K68" s="38"/>
+      <c r="L68" s="38"/>
     </row>
     <row r="69" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J69" s="34"/>
-      <c r="K69" s="34"/>
-      <c r="L69" s="34"/>
+      <c r="J69" s="38"/>
+      <c r="K69" s="38"/>
+      <c r="L69" s="38"/>
     </row>
     <row r="70" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J70" s="34"/>
-      <c r="K70" s="34"/>
-      <c r="L70" s="34"/>
+      <c r="J70" s="38"/>
+      <c r="K70" s="38"/>
+      <c r="L70" s="38"/>
     </row>
     <row r="71" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J71" s="34"/>
-      <c r="K71" s="34"/>
-      <c r="L71" s="34"/>
+      <c r="J71" s="38"/>
+      <c r="K71" s="38"/>
+      <c r="L71" s="38"/>
     </row>
     <row r="72" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J72" s="34"/>
-      <c r="K72" s="34"/>
-      <c r="L72" s="34"/>
+      <c r="J72" s="38"/>
+      <c r="K72" s="38"/>
+      <c r="L72" s="38"/>
     </row>
     <row r="73" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J73" s="34"/>
-      <c r="K73" s="34"/>
-      <c r="L73" s="34"/>
+      <c r="J73" s="38"/>
+      <c r="K73" s="38"/>
+      <c r="L73" s="38"/>
     </row>
     <row r="74" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J74" s="34"/>
-      <c r="K74" s="34"/>
-      <c r="L74" s="34"/>
+      <c r="J74" s="38"/>
+      <c r="K74" s="38"/>
+      <c r="L74" s="38"/>
     </row>
     <row r="75" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J75" s="34"/>
-      <c r="K75" s="34"/>
-      <c r="L75" s="34"/>
+      <c r="J75" s="38"/>
+      <c r="K75" s="38"/>
+      <c r="L75" s="38"/>
     </row>
     <row r="76" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J76" s="34"/>
-      <c r="K76" s="34"/>
-      <c r="L76" s="34"/>
+      <c r="J76" s="38"/>
+      <c r="K76" s="38"/>
+      <c r="L76" s="38"/>
     </row>
     <row r="77" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J77" s="34"/>
-      <c r="K77" s="34"/>
-      <c r="L77" s="34"/>
+      <c r="J77" s="38"/>
+      <c r="K77" s="38"/>
+      <c r="L77" s="38"/>
     </row>
     <row r="78" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J78" s="34"/>
-      <c r="K78" s="34"/>
-      <c r="L78" s="34"/>
+      <c r="J78" s="38"/>
+      <c r="K78" s="38"/>
+      <c r="L78" s="38"/>
     </row>
     <row r="79" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J79" s="34"/>
-      <c r="K79" s="34"/>
-      <c r="L79" s="34"/>
+      <c r="J79" s="38"/>
+      <c r="K79" s="38"/>
+      <c r="L79" s="38"/>
     </row>
     <row r="80" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J80" s="34"/>
-      <c r="K80" s="34"/>
-      <c r="L80" s="34"/>
+      <c r="J80" s="38"/>
+      <c r="K80" s="38"/>
+      <c r="L80" s="38"/>
     </row>
     <row r="81" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J81" s="34"/>
-      <c r="K81" s="34"/>
-      <c r="L81" s="34"/>
+      <c r="J81" s="38"/>
+      <c r="K81" s="38"/>
+      <c r="L81" s="38"/>
     </row>
     <row r="82" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J82" s="34"/>
-      <c r="K82" s="34"/>
-      <c r="L82" s="34"/>
+      <c r="J82" s="38"/>
+      <c r="K82" s="38"/>
+      <c r="L82" s="38"/>
     </row>
     <row r="83" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J83" s="34"/>
-      <c r="K83" s="34"/>
-      <c r="L83" s="34"/>
+      <c r="J83" s="38"/>
+      <c r="K83" s="38"/>
+      <c r="L83" s="38"/>
     </row>
     <row r="84" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J84" s="34"/>
-      <c r="K84" s="34"/>
-      <c r="L84" s="34"/>
+      <c r="J84" s="38"/>
+      <c r="K84" s="38"/>
+      <c r="L84" s="38"/>
     </row>
     <row r="85" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J85" s="34"/>
-      <c r="K85" s="34"/>
-      <c r="L85" s="34"/>
+      <c r="J85" s="38"/>
+      <c r="K85" s="38"/>
+      <c r="L85" s="38"/>
     </row>
     <row r="86" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J86" s="34"/>
-      <c r="K86" s="34"/>
-      <c r="L86" s="34"/>
+      <c r="J86" s="38"/>
+      <c r="K86" s="38"/>
+      <c r="L86" s="38"/>
     </row>
     <row r="87" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J87" s="34"/>
-      <c r="K87" s="34"/>
-      <c r="L87" s="34"/>
+      <c r="J87" s="38"/>
+      <c r="K87" s="38"/>
+      <c r="L87" s="38"/>
     </row>
     <row r="88" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J88" s="34"/>
-      <c r="K88" s="34"/>
-      <c r="L88" s="34"/>
+      <c r="J88" s="38"/>
+      <c r="K88" s="38"/>
+      <c r="L88" s="38"/>
     </row>
     <row r="89" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J89" s="34"/>
-      <c r="K89" s="34"/>
-      <c r="L89" s="34"/>
+      <c r="J89" s="38"/>
+      <c r="K89" s="38"/>
+      <c r="L89" s="38"/>
     </row>
     <row r="90" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J90" s="34"/>
-      <c r="K90" s="34"/>
-      <c r="L90" s="34"/>
+      <c r="J90" s="38"/>
+      <c r="K90" s="38"/>
+      <c r="L90" s="38"/>
     </row>
     <row r="91" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J91" s="34"/>
-      <c r="K91" s="34"/>
-      <c r="L91" s="34"/>
+      <c r="J91" s="38"/>
+      <c r="K91" s="38"/>
+      <c r="L91" s="38"/>
     </row>
     <row r="92" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J92" s="34"/>
-      <c r="K92" s="34"/>
-      <c r="L92" s="34"/>
+      <c r="J92" s="38"/>
+      <c r="K92" s="38"/>
+      <c r="L92" s="38"/>
     </row>
     <row r="93" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J93" s="34"/>
-      <c r="K93" s="34"/>
-      <c r="L93" s="34"/>
+      <c r="J93" s="38"/>
+      <c r="K93" s="38"/>
+      <c r="L93" s="38"/>
     </row>
     <row r="94" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J94" s="34"/>
-      <c r="K94" s="34"/>
-      <c r="L94" s="34"/>
+      <c r="J94" s="38"/>
+      <c r="K94" s="38"/>
+      <c r="L94" s="38"/>
     </row>
     <row r="95" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J95" s="34"/>
-      <c r="K95" s="34"/>
-      <c r="L95" s="34"/>
+      <c r="J95" s="38"/>
+      <c r="K95" s="38"/>
+      <c r="L95" s="38"/>
     </row>
     <row r="96" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J96" s="34"/>
-      <c r="K96" s="34"/>
-      <c r="L96" s="34"/>
+      <c r="J96" s="38"/>
+      <c r="K96" s="38"/>
+      <c r="L96" s="38"/>
     </row>
     <row r="97" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J97" s="34"/>
-      <c r="K97" s="34"/>
-      <c r="L97" s="34"/>
+      <c r="J97" s="38"/>
+      <c r="K97" s="38"/>
+      <c r="L97" s="38"/>
     </row>
     <row r="98" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J98" s="34"/>
-      <c r="K98" s="34"/>
-      <c r="L98" s="34"/>
+      <c r="J98" s="38"/>
+      <c r="K98" s="38"/>
+      <c r="L98" s="38"/>
     </row>
     <row r="99" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J99" s="34"/>
-      <c r="K99" s="34"/>
-      <c r="L99" s="34"/>
+      <c r="J99" s="38"/>
+      <c r="K99" s="38"/>
+      <c r="L99" s="38"/>
     </row>
     <row r="100" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J100" s="34"/>
-      <c r="K100" s="34"/>
-      <c r="L100" s="34"/>
+      <c r="J100" s="38"/>
+      <c r="K100" s="38"/>
+      <c r="L100" s="38"/>
     </row>
     <row r="101" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J101" s="34"/>
-      <c r="K101" s="34"/>
-      <c r="L101" s="34"/>
+      <c r="J101" s="38"/>
+      <c r="K101" s="38"/>
+      <c r="L101" s="38"/>
     </row>
     <row r="102" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J102" s="34"/>
-      <c r="K102" s="34"/>
-      <c r="L102" s="34"/>
+      <c r="J102" s="38"/>
+      <c r="K102" s="38"/>
+      <c r="L102" s="38"/>
     </row>
     <row r="103" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J103" s="34"/>
-      <c r="K103" s="34"/>
-      <c r="L103" s="34"/>
+      <c r="J103" s="38"/>
+      <c r="K103" s="38"/>
+      <c r="L103" s="38"/>
     </row>
     <row r="104" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J104" s="34"/>
-      <c r="K104" s="34"/>
-      <c r="L104" s="34"/>
+      <c r="J104" s="38"/>
+      <c r="K104" s="38"/>
+      <c r="L104" s="38"/>
     </row>
     <row r="105" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J105" s="34"/>
-      <c r="K105" s="34"/>
-      <c r="L105" s="34"/>
+      <c r="J105" s="38"/>
+      <c r="K105" s="38"/>
+      <c r="L105" s="38"/>
     </row>
     <row r="106" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J106" s="34"/>
-      <c r="K106" s="34"/>
-      <c r="L106" s="34"/>
+      <c r="J106" s="38"/>
+      <c r="K106" s="38"/>
+      <c r="L106" s="38"/>
     </row>
     <row r="107" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J107" s="34"/>
-      <c r="K107" s="34"/>
-      <c r="L107" s="34"/>
+      <c r="J107" s="38"/>
+      <c r="K107" s="38"/>
+      <c r="L107" s="38"/>
     </row>
     <row r="108" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J108" s="34"/>
-      <c r="K108" s="34"/>
-      <c r="L108" s="34"/>
+      <c r="J108" s="38"/>
+      <c r="K108" s="38"/>
+      <c r="L108" s="38"/>
     </row>
     <row r="109" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J109" s="34"/>
-      <c r="K109" s="34"/>
-      <c r="L109" s="34"/>
+      <c r="J109" s="38"/>
+      <c r="K109" s="38"/>
+      <c r="L109" s="38"/>
     </row>
     <row r="110" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J110" s="34"/>
-      <c r="K110" s="34"/>
-      <c r="L110" s="34"/>
+      <c r="J110" s="38"/>
+      <c r="K110" s="38"/>
+      <c r="L110" s="38"/>
     </row>
     <row r="111" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J111" s="34"/>
-      <c r="K111" s="34"/>
-      <c r="L111" s="34"/>
+      <c r="J111" s="38"/>
+      <c r="K111" s="38"/>
+      <c r="L111" s="38"/>
     </row>
     <row r="112" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J112" s="34"/>
-      <c r="K112" s="34"/>
-      <c r="L112" s="34"/>
+      <c r="J112" s="38"/>
+      <c r="K112" s="38"/>
+      <c r="L112" s="38"/>
     </row>
     <row r="113" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J113" s="34"/>
-      <c r="K113" s="34"/>
-      <c r="L113" s="34"/>
+      <c r="J113" s="38"/>
+      <c r="K113" s="38"/>
+      <c r="L113" s="38"/>
     </row>
     <row r="114" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J114" s="34"/>
-      <c r="K114" s="34"/>
-      <c r="L114" s="34"/>
+      <c r="J114" s="38"/>
+      <c r="K114" s="38"/>
+      <c r="L114" s="38"/>
     </row>
     <row r="115" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J115" s="34"/>
-      <c r="K115" s="34"/>
-      <c r="L115" s="34"/>
+      <c r="J115" s="38"/>
+      <c r="K115" s="38"/>
+      <c r="L115" s="38"/>
     </row>
     <row r="116" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J116" s="34"/>
-      <c r="K116" s="34"/>
-      <c r="L116" s="34"/>
+      <c r="J116" s="38"/>
+      <c r="K116" s="38"/>
+      <c r="L116" s="38"/>
     </row>
     <row r="117" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J117" s="34"/>
-      <c r="K117" s="34"/>
-      <c r="L117" s="34"/>
+      <c r="J117" s="38"/>
+      <c r="K117" s="38"/>
+      <c r="L117" s="38"/>
     </row>
     <row r="118" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J118" s="34"/>
-      <c r="K118" s="34"/>
-      <c r="L118" s="34"/>
+      <c r="J118" s="38"/>
+      <c r="K118" s="38"/>
+      <c r="L118" s="38"/>
     </row>
     <row r="119" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J119" s="34"/>
-      <c r="K119" s="34"/>
-      <c r="L119" s="34"/>
+      <c r="J119" s="38"/>
+      <c r="K119" s="38"/>
+      <c r="L119" s="38"/>
     </row>
     <row r="120" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J120" s="34"/>
-      <c r="K120" s="34"/>
-      <c r="L120" s="34"/>
+      <c r="J120" s="38"/>
+      <c r="K120" s="38"/>
+      <c r="L120" s="38"/>
     </row>
     <row r="121" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J121" s="34"/>
-      <c r="K121" s="34"/>
-      <c r="L121" s="34"/>
+      <c r="J121" s="38"/>
+      <c r="K121" s="38"/>
+      <c r="L121" s="38"/>
     </row>
     <row r="122" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J122" s="34"/>
-      <c r="K122" s="34"/>
-      <c r="L122" s="34"/>
+      <c r="J122" s="38"/>
+      <c r="K122" s="38"/>
+      <c r="L122" s="38"/>
     </row>
     <row r="123" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J123" s="34"/>
-      <c r="K123" s="34"/>
-      <c r="L123" s="34"/>
+      <c r="J123" s="38"/>
+      <c r="K123" s="38"/>
+      <c r="L123" s="38"/>
     </row>
     <row r="124" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J124" s="34"/>
-      <c r="K124" s="34"/>
-      <c r="L124" s="34"/>
+      <c r="J124" s="38"/>
+      <c r="K124" s="38"/>
+      <c r="L124" s="38"/>
     </row>
     <row r="125" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J125" s="34"/>
-      <c r="K125" s="34"/>
-      <c r="L125" s="34"/>
+      <c r="J125" s="38"/>
+      <c r="K125" s="38"/>
+      <c r="L125" s="38"/>
     </row>
     <row r="126" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J126" s="34"/>
-      <c r="K126" s="34"/>
-      <c r="L126" s="34"/>
+      <c r="J126" s="38"/>
+      <c r="K126" s="38"/>
+      <c r="L126" s="38"/>
     </row>
     <row r="127" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J127" s="34"/>
-      <c r="K127" s="34"/>
-      <c r="L127" s="34"/>
+      <c r="J127" s="38"/>
+      <c r="K127" s="38"/>
+      <c r="L127" s="38"/>
     </row>
     <row r="128" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J128" s="34"/>
-      <c r="K128" s="34"/>
-      <c r="L128" s="34"/>
+      <c r="J128" s="38"/>
+      <c r="K128" s="38"/>
+      <c r="L128" s="38"/>
     </row>
     <row r="129" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J129" s="34"/>
-      <c r="K129" s="34"/>
-      <c r="L129" s="34"/>
+      <c r="J129" s="38"/>
+      <c r="K129" s="38"/>
+      <c r="L129" s="38"/>
     </row>
     <row r="130" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J130" s="34"/>
-      <c r="K130" s="34"/>
-      <c r="L130" s="34"/>
+      <c r="J130" s="38"/>
+      <c r="K130" s="38"/>
+      <c r="L130" s="38"/>
     </row>
     <row r="131" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J131" s="34"/>
-      <c r="K131" s="34"/>
-      <c r="L131" s="34"/>
+      <c r="J131" s="38"/>
+      <c r="K131" s="38"/>
+      <c r="L131" s="38"/>
     </row>
     <row r="132" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J132" s="34"/>
-      <c r="K132" s="34"/>
-      <c r="L132" s="34"/>
+      <c r="J132" s="38"/>
+      <c r="K132" s="38"/>
+      <c r="L132" s="38"/>
     </row>
     <row r="133" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J133" s="34"/>
-      <c r="K133" s="34"/>
-      <c r="L133" s="34"/>
+      <c r="J133" s="38"/>
+      <c r="K133" s="38"/>
+      <c r="L133" s="38"/>
     </row>
     <row r="134" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J134" s="34"/>
-      <c r="K134" s="34"/>
-      <c r="L134" s="34"/>
+      <c r="J134" s="38"/>
+      <c r="K134" s="38"/>
+      <c r="L134" s="38"/>
     </row>
     <row r="135" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J135" s="34"/>
-      <c r="K135" s="34"/>
-      <c r="L135" s="34"/>
+      <c r="J135" s="38"/>
+      <c r="K135" s="38"/>
+      <c r="L135" s="38"/>
     </row>
     <row r="136" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J136" s="34"/>
-      <c r="K136" s="34"/>
-      <c r="L136" s="34"/>
+      <c r="J136" s="38"/>
+      <c r="K136" s="38"/>
+      <c r="L136" s="38"/>
     </row>
     <row r="137" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J137" s="34"/>
-      <c r="K137" s="34"/>
-      <c r="L137" s="34"/>
+      <c r="J137" s="38"/>
+      <c r="K137" s="38"/>
+      <c r="L137" s="38"/>
     </row>
     <row r="138" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J138" s="34"/>
-      <c r="K138" s="34"/>
-      <c r="L138" s="34"/>
+      <c r="J138" s="38"/>
+      <c r="K138" s="38"/>
+      <c r="L138" s="38"/>
     </row>
     <row r="139" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J139" s="34"/>
-      <c r="K139" s="34"/>
-      <c r="L139" s="34"/>
+      <c r="J139" s="38"/>
+      <c r="K139" s="38"/>
+      <c r="L139" s="38"/>
     </row>
     <row r="140" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J140" s="34"/>
-      <c r="K140" s="34"/>
-      <c r="L140" s="34"/>
+      <c r="J140" s="38"/>
+      <c r="K140" s="38"/>
+      <c r="L140" s="38"/>
     </row>
     <row r="141" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J141" s="34"/>
-      <c r="K141" s="34"/>
-      <c r="L141" s="34"/>
+      <c r="J141" s="38"/>
+      <c r="K141" s="38"/>
+      <c r="L141" s="38"/>
     </row>
     <row r="142" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J142" s="34"/>
-      <c r="K142" s="34"/>
-      <c r="L142" s="34"/>
+      <c r="J142" s="38"/>
+      <c r="K142" s="38"/>
+      <c r="L142" s="38"/>
     </row>
     <row r="143" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J143" s="34"/>
-      <c r="K143" s="34"/>
-      <c r="L143" s="34"/>
+      <c r="J143" s="38"/>
+      <c r="K143" s="38"/>
+      <c r="L143" s="38"/>
     </row>
     <row r="144" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J144" s="34"/>
-      <c r="K144" s="34"/>
-      <c r="L144" s="34"/>
+      <c r="J144" s="38"/>
+      <c r="K144" s="38"/>
+      <c r="L144" s="38"/>
     </row>
     <row r="145" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J145" s="34"/>
-      <c r="K145" s="34"/>
-      <c r="L145" s="34"/>
+      <c r="J145" s="38"/>
+      <c r="K145" s="38"/>
+      <c r="L145" s="38"/>
     </row>
     <row r="146" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J146" s="34"/>
-      <c r="K146" s="34"/>
-      <c r="L146" s="34"/>
+      <c r="J146" s="38"/>
+      <c r="K146" s="38"/>
+      <c r="L146" s="38"/>
     </row>
     <row r="147" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J147" s="34"/>
-      <c r="K147" s="34"/>
-      <c r="L147" s="34"/>
+      <c r="J147" s="38"/>
+      <c r="K147" s="38"/>
+      <c r="L147" s="38"/>
     </row>
     <row r="148" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J148" s="34"/>
-      <c r="K148" s="34"/>
-      <c r="L148" s="34"/>
+      <c r="J148" s="38"/>
+      <c r="K148" s="38"/>
+      <c r="L148" s="38"/>
     </row>
     <row r="149" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J149" s="34"/>
-      <c r="K149" s="34"/>
-      <c r="L149" s="34"/>
+      <c r="J149" s="38"/>
+      <c r="K149" s="38"/>
+      <c r="L149" s="38"/>
     </row>
     <row r="150" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J150" s="34"/>
-      <c r="K150" s="34"/>
-      <c r="L150" s="34"/>
+      <c r="J150" s="38"/>
+      <c r="K150" s="38"/>
+      <c r="L150" s="38"/>
     </row>
     <row r="151" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J151" s="34"/>
-      <c r="K151" s="34"/>
-      <c r="L151" s="34"/>
+      <c r="J151" s="38"/>
+      <c r="K151" s="38"/>
+      <c r="L151" s="38"/>
     </row>
     <row r="152" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J152" s="34"/>
-      <c r="K152" s="34"/>
-      <c r="L152" s="34"/>
+      <c r="J152" s="38"/>
+      <c r="K152" s="38"/>
+      <c r="L152" s="38"/>
     </row>
     <row r="153" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J153" s="34"/>
-      <c r="K153" s="34"/>
-      <c r="L153" s="34"/>
+      <c r="J153" s="38"/>
+      <c r="K153" s="38"/>
+      <c r="L153" s="38"/>
     </row>
     <row r="154" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J154" s="34"/>
-      <c r="K154" s="34"/>
-      <c r="L154" s="34"/>
+      <c r="J154" s="38"/>
+      <c r="K154" s="38"/>
+      <c r="L154" s="38"/>
     </row>
     <row r="155" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J155" s="34"/>
-      <c r="K155" s="34"/>
-      <c r="L155" s="34"/>
+      <c r="J155" s="38"/>
+      <c r="K155" s="38"/>
+      <c r="L155" s="38"/>
     </row>
     <row r="156" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J156" s="34"/>
-      <c r="K156" s="34"/>
-      <c r="L156" s="34"/>
+      <c r="J156" s="38"/>
+      <c r="K156" s="38"/>
+      <c r="L156" s="38"/>
     </row>
     <row r="157" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J157" s="34"/>
-      <c r="K157" s="34"/>
-      <c r="L157" s="34"/>
+      <c r="J157" s="38"/>
+      <c r="K157" s="38"/>
+      <c r="L157" s="38"/>
     </row>
     <row r="158" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J158" s="34"/>
-      <c r="K158" s="34"/>
-      <c r="L158" s="34"/>
+      <c r="J158" s="38"/>
+      <c r="K158" s="38"/>
+      <c r="L158" s="38"/>
     </row>
     <row r="159" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J159" s="34"/>
-      <c r="K159" s="34"/>
-      <c r="L159" s="34"/>
+      <c r="J159" s="38"/>
+      <c r="K159" s="38"/>
+      <c r="L159" s="38"/>
     </row>
     <row r="160" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J160" s="34"/>
-      <c r="K160" s="34"/>
-      <c r="L160" s="34"/>
+      <c r="J160" s="38"/>
+      <c r="K160" s="38"/>
+      <c r="L160" s="38"/>
     </row>
     <row r="161" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J161" s="34"/>
-      <c r="K161" s="34"/>
-      <c r="L161" s="34"/>
+      <c r="J161" s="38"/>
+      <c r="K161" s="38"/>
+      <c r="L161" s="38"/>
     </row>
     <row r="162" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J162" s="34"/>
-      <c r="K162" s="34"/>
-      <c r="L162" s="34"/>
+      <c r="J162" s="38"/>
+      <c r="K162" s="38"/>
+      <c r="L162" s="38"/>
     </row>
     <row r="163" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J163" s="34"/>
-      <c r="K163" s="34"/>
-      <c r="L163" s="34"/>
+      <c r="J163" s="38"/>
+      <c r="K163" s="38"/>
+      <c r="L163" s="38"/>
     </row>
     <row r="164" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J164" s="34"/>
-      <c r="K164" s="34"/>
-      <c r="L164" s="34"/>
+      <c r="J164" s="38"/>
+      <c r="K164" s="38"/>
+      <c r="L164" s="38"/>
     </row>
     <row r="165" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J165" s="34"/>
-      <c r="K165" s="34"/>
-      <c r="L165" s="34"/>
+      <c r="J165" s="38"/>
+      <c r="K165" s="38"/>
+      <c r="L165" s="38"/>
     </row>
     <row r="166" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J166" s="34"/>
-      <c r="K166" s="34"/>
-      <c r="L166" s="34"/>
+      <c r="J166" s="38"/>
+      <c r="K166" s="38"/>
+      <c r="L166" s="38"/>
     </row>
     <row r="167" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J167" s="34"/>
-      <c r="K167" s="34"/>
-      <c r="L167" s="34"/>
+      <c r="J167" s="38"/>
+      <c r="K167" s="38"/>
+      <c r="L167" s="38"/>
     </row>
     <row r="168" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J168" s="34"/>
-      <c r="K168" s="34"/>
-      <c r="L168" s="34"/>
+      <c r="J168" s="38"/>
+      <c r="K168" s="38"/>
+      <c r="L168" s="38"/>
     </row>
     <row r="169" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J169" s="34"/>
-      <c r="K169" s="34"/>
-      <c r="L169" s="34"/>
+      <c r="J169" s="38"/>
+      <c r="K169" s="38"/>
+      <c r="L169" s="38"/>
     </row>
     <row r="170" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J170" s="34"/>
-      <c r="K170" s="34"/>
-      <c r="L170" s="34"/>
+      <c r="J170" s="38"/>
+      <c r="K170" s="38"/>
+      <c r="L170" s="38"/>
     </row>
     <row r="171" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J171" s="34"/>
-      <c r="K171" s="34"/>
-      <c r="L171" s="34"/>
+      <c r="J171" s="38"/>
+      <c r="K171" s="38"/>
+      <c r="L171" s="38"/>
     </row>
     <row r="172" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J172" s="34"/>
-      <c r="K172" s="34"/>
-      <c r="L172" s="34"/>
+      <c r="J172" s="38"/>
+      <c r="K172" s="38"/>
+      <c r="L172" s="38"/>
     </row>
     <row r="173" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J173" s="34"/>
-      <c r="K173" s="34"/>
-      <c r="L173" s="34"/>
+      <c r="J173" s="38"/>
+      <c r="K173" s="38"/>
+      <c r="L173" s="38"/>
     </row>
     <row r="174" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J174" s="34"/>
-      <c r="K174" s="34"/>
-      <c r="L174" s="34"/>
+      <c r="J174" s="38"/>
+      <c r="K174" s="38"/>
+      <c r="L174" s="38"/>
     </row>
     <row r="175" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J175" s="34"/>
-      <c r="K175" s="34"/>
-      <c r="L175" s="34"/>
+      <c r="J175" s="38"/>
+      <c r="K175" s="38"/>
+      <c r="L175" s="38"/>
     </row>
     <row r="176" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J176" s="34"/>
-      <c r="K176" s="34"/>
-      <c r="L176" s="34"/>
+      <c r="J176" s="38"/>
+      <c r="K176" s="38"/>
+      <c r="L176" s="38"/>
     </row>
     <row r="177" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J177" s="34"/>
-      <c r="K177" s="34"/>
-      <c r="L177" s="34"/>
+      <c r="J177" s="38"/>
+      <c r="K177" s="38"/>
+      <c r="L177" s="38"/>
     </row>
     <row r="178" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J178" s="34"/>
-      <c r="K178" s="34"/>
-      <c r="L178" s="34"/>
+      <c r="J178" s="38"/>
+      <c r="K178" s="38"/>
+      <c r="L178" s="38"/>
     </row>
     <row r="179" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J179" s="34"/>
-      <c r="K179" s="34"/>
-      <c r="L179" s="34"/>
+      <c r="J179" s="38"/>
+      <c r="K179" s="38"/>
+      <c r="L179" s="38"/>
     </row>
     <row r="180" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J180" s="34"/>
-      <c r="K180" s="34"/>
-      <c r="L180" s="34"/>
+      <c r="J180" s="38"/>
+      <c r="K180" s="38"/>
+      <c r="L180" s="38"/>
     </row>
     <row r="181" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J181" s="34"/>
-      <c r="K181" s="34"/>
-      <c r="L181" s="34"/>
+      <c r="J181" s="38"/>
+      <c r="K181" s="38"/>
+      <c r="L181" s="38"/>
     </row>
     <row r="182" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J182" s="34"/>
-      <c r="K182" s="34"/>
-      <c r="L182" s="34"/>
+      <c r="J182" s="38"/>
+      <c r="K182" s="38"/>
+      <c r="L182" s="38"/>
     </row>
     <row r="183" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J183" s="34"/>
-      <c r="K183" s="34"/>
-      <c r="L183" s="34"/>
+      <c r="J183" s="38"/>
+      <c r="K183" s="38"/>
+      <c r="L183" s="38"/>
     </row>
     <row r="184" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J184" s="34"/>
-      <c r="K184" s="34"/>
-      <c r="L184" s="34"/>
+      <c r="J184" s="38"/>
+      <c r="K184" s="38"/>
+      <c r="L184" s="38"/>
     </row>
     <row r="185" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J185" s="34"/>
-      <c r="K185" s="34"/>
-      <c r="L185" s="34"/>
+      <c r="J185" s="38"/>
+      <c r="K185" s="38"/>
+      <c r="L185" s="38"/>
     </row>
     <row r="186" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J186" s="34"/>
-      <c r="K186" s="34"/>
-      <c r="L186" s="34"/>
+      <c r="J186" s="38"/>
+      <c r="K186" s="38"/>
+      <c r="L186" s="38"/>
     </row>
     <row r="187" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J187" s="34"/>
-      <c r="K187" s="34"/>
-      <c r="L187" s="34"/>
+      <c r="J187" s="38"/>
+      <c r="K187" s="38"/>
+      <c r="L187" s="38"/>
     </row>
     <row r="188" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J188" s="34"/>
-      <c r="K188" s="34"/>
-      <c r="L188" s="34"/>
+      <c r="J188" s="38"/>
+      <c r="K188" s="38"/>
+      <c r="L188" s="38"/>
     </row>
     <row r="189" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J189" s="34"/>
-      <c r="K189" s="34"/>
-      <c r="L189" s="34"/>
+      <c r="J189" s="38"/>
+      <c r="K189" s="38"/>
+      <c r="L189" s="38"/>
     </row>
     <row r="190" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J190" s="34"/>
-      <c r="K190" s="34"/>
-      <c r="L190" s="34"/>
+      <c r="J190" s="38"/>
+      <c r="K190" s="38"/>
+      <c r="L190" s="38"/>
     </row>
     <row r="191" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J191" s="34"/>
-      <c r="K191" s="34"/>
-      <c r="L191" s="34"/>
+      <c r="J191" s="38"/>
+      <c r="K191" s="38"/>
+      <c r="L191" s="38"/>
     </row>
     <row r="192" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J192" s="34"/>
-      <c r="K192" s="34"/>
-      <c r="L192" s="34"/>
+      <c r="J192" s="38"/>
+      <c r="K192" s="38"/>
+      <c r="L192" s="38"/>
     </row>
     <row r="193" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J193" s="34"/>
-      <c r="K193" s="34"/>
-      <c r="L193" s="34"/>
+      <c r="J193" s="38"/>
+      <c r="K193" s="38"/>
+      <c r="L193" s="38"/>
     </row>
     <row r="194" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J194" s="34"/>
-      <c r="K194" s="34"/>
-      <c r="L194" s="34"/>
+      <c r="J194" s="38"/>
+      <c r="K194" s="38"/>
+      <c r="L194" s="38"/>
     </row>
     <row r="195" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J195" s="34"/>
-      <c r="K195" s="34"/>
-      <c r="L195" s="34"/>
+      <c r="J195" s="38"/>
+      <c r="K195" s="38"/>
+      <c r="L195" s="38"/>
     </row>
     <row r="196" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J196" s="34"/>
-      <c r="K196" s="34"/>
-      <c r="L196" s="34"/>
+      <c r="J196" s="38"/>
+      <c r="K196" s="38"/>
+      <c r="L196" s="38"/>
     </row>
     <row r="197" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J197" s="34"/>
-      <c r="K197" s="34"/>
-      <c r="L197" s="34"/>
+      <c r="J197" s="38"/>
+      <c r="K197" s="38"/>
+      <c r="L197" s="38"/>
     </row>
     <row r="198" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J198" s="34"/>
-      <c r="K198" s="34"/>
-      <c r="L198" s="34"/>
+      <c r="J198" s="38"/>
+      <c r="K198" s="38"/>
+      <c r="L198" s="38"/>
     </row>
     <row r="199" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J199" s="34"/>
-      <c r="K199" s="34"/>
-      <c r="L199" s="34"/>
+      <c r="J199" s="38"/>
+      <c r="K199" s="38"/>
+      <c r="L199" s="38"/>
     </row>
     <row r="200" spans="10:12" x14ac:dyDescent="0.3">
-      <c r="J200" s="34"/>
-      <c r="K200" s="34"/>
-      <c r="L200" s="34"/>
+      <c r="J200" s="38"/>
+      <c r="K200" s="38"/>
+      <c r="L200" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>